<commit_message>
Kyoto Ink V3.3 célképek átvétele és első költségfrissítés
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R7f95b05598c64e3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="R5f78fc30ecaa4ca6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="Rbbfa7d80ad274139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R985b6d9d809d453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R7bee71ea53fa4dc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="Rb15119f63f9344fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R907eaa7f4d524918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R9b1fc3272e8548cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1108,10 +1108,10 @@
       </x:c>
       <x:c r="B7" s="18" t="n">
         <x:f>SUM('Elemregiszter'!U2:U160)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>Aktuális, teljes tartalom</x:v>
+        <x:v>V3.3 célátvétel: +210 000 Ft; 159 költségsor; minden új ár becslés</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -1120,7 +1120,7 @@
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f>SUM('Elemregiszter'!AH2:AH160)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
         <x:v>Még nincs optimalizált változat; egyelőre a fővel azonos</x:v>
@@ -1132,7 +1132,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>B7-B5</x:f>
-        <x:v>2083350</x:v>
+        <x:v>2293350</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -1144,7 +1144,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>B8-B5</x:f>
-        <x:v>2083350</x:v>
+        <x:v>2293350</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>B7-B11-B12</x:f>
-        <x:v>18661080</x:v>
+        <x:v>18871080</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>Minden nem igazolt ár</x:v>
@@ -1302,11 +1302,11 @@
       </x:c>
       <x:c r="B25" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$B$2:$B$160,A25)</x:f>
-        <x:v>3051190</x:v>
+        <x:v>3321190</x:v>
       </x:c>
       <x:c r="C25" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$B$2:$B$160,A25)</x:f>
-        <x:v>3051190</x:v>
+        <x:v>3321190</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
@@ -1471,11 +1471,11 @@
       </x:c>
       <x:c r="B38" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$B$2:$B$160,A38)</x:f>
-        <x:v>375000</x:v>
+        <x:v>315000</x:v>
       </x:c>
       <x:c r="C38" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$B$2:$B$160,A38)</x:f>
-        <x:v>375000</x:v>
+        <x:v>315000</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="30" customHeight="1">
@@ -1570,11 +1570,11 @@
       </x:c>
       <x:c r="B47" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$G$2:$G$160,A47)</x:f>
-        <x:v>4760000</x:v>
+        <x:v>4890000</x:v>
       </x:c>
       <x:c r="C47" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$G$2:$G$160,A47)</x:f>
-        <x:v>4760000</x:v>
+        <x:v>4890000</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="30" customHeight="1">
@@ -1648,11 +1648,11 @@
       </x:c>
       <x:c r="B53" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$G$2:$G$160,A53)</x:f>
-        <x:v>350000</x:v>
+        <x:v>490000</x:v>
       </x:c>
       <x:c r="C53" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$G$2:$G$160,A53)</x:f>
-        <x:v>350000</x:v>
+        <x:v>490000</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="30" customHeight="1">
@@ -1700,11 +1700,11 @@
       </x:c>
       <x:c r="B57" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$G$2:$G$160,A57)</x:f>
-        <x:v>465000</x:v>
+        <x:v>405000</x:v>
       </x:c>
       <x:c r="C57" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$G$2:$G$160,A57)</x:f>
-        <x:v>465000</x:v>
+        <x:v>405000</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="30" customHeight="1">
@@ -1773,11 +1773,11 @@
       </x:c>
       <x:c r="B64" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$F$2:$F$160,A64)</x:f>
-        <x:v>11248350</x:v>
+        <x:v>11458350</x:v>
       </x:c>
       <x:c r="C64" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$F$2:$F$160,A64)</x:f>
-        <x:v>11248350</x:v>
+        <x:v>11458350</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="30" customHeight="1">
@@ -1807,11 +1807,11 @@
       </x:c>
       <x:c r="B68" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$AC$2:$AC$160,A68)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
       <x:c r="C68" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$AC$2:$AC$160,A68)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -5515,7 +5515,7 @@
         <x:v>KI-030</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>Cam02 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
         <x:v>03a</x:v>
@@ -5554,7 +5554,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q31" s="20" t="n">
-        <x:v>310000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="R31" s="20" t="n">
         <x:v>0</x:v>
@@ -5567,13 +5567,13 @@
       </x:c>
       <x:c r="U31" s="21" t="n">
         <x:f>O31*Q31+SUM(R31:T31)</x:f>
-        <x:v>310000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="V31" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W31" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03a</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X31" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -5600,17 +5600,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF31" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>W01 V3.3 panelmező, grafikus torony: nagyobb folytonos grafika; 3600×2880 tervezési befoglaló</x:v>
       </x:c>
       <x:c r="AG31" s="20" t="n">
-        <x:v>310000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="AH31" s="21" t="n">
         <x:f>O31*AG31+SUM(R31:T31)</x:f>
-        <x:v>310000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="AI31" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ31" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -5636,7 +5636,7 @@
         <x:v>KI-031</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>Cam02 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
         <x:v>03a</x:v>
@@ -5675,7 +5675,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q32" s="20" t="n">
-        <x:v>210000</x:v>
+        <x:v>260000</x:v>
       </x:c>
       <x:c r="R32" s="20" t="n">
         <x:v>0</x:v>
@@ -5688,13 +5688,13 @@
       </x:c>
       <x:c r="U32" s="21" t="n">
         <x:f>O32*Q32+SUM(R32:T32)</x:f>
-        <x:v>210000</x:v>
+        <x:v>260000</x:v>
       </x:c>
       <x:c r="V32" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W32" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03a</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X32" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -5721,17 +5721,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF32" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>W01 V3.3 folytonos alsó tároló: 3300×400×400, 5 front</x:v>
       </x:c>
       <x:c r="AG32" s="20" t="n">
-        <x:v>210000</x:v>
+        <x:v>260000</x:v>
       </x:c>
       <x:c r="AH32" s="21" t="n">
         <x:f>O32*AG32+SUM(R32:T32)</x:f>
-        <x:v>210000</x:v>
+        <x:v>260000</x:v>
       </x:c>
       <x:c r="AI32" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ32" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -6362,7 +6362,7 @@
         <x:v>KI-037</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>Cam02 v1; Cam12 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
         <x:v>03c</x:v>
@@ -6401,7 +6401,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q38" s="20" t="n">
-        <x:v>150000</x:v>
+        <x:v>105000</x:v>
       </x:c>
       <x:c r="R38" s="20" t="n">
         <x:v>0</x:v>
@@ -6414,13 +6414,13 @@
       </x:c>
       <x:c r="U38" s="21" t="n">
         <x:f>O38*Q38+SUM(R38:T38)</x:f>
-        <x:v>150000</x:v>
+        <x:v>105000</x:v>
       </x:c>
       <x:c r="V38" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W38" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03c</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X38" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -6447,17 +6447,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF38" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>Egyedi CF-01 grafit laminált dobozasztal 700×450×350 mm</x:v>
       </x:c>
       <x:c r="AG38" s="20" t="n">
-        <x:v>150000</x:v>
+        <x:v>105000</x:v>
       </x:c>
       <x:c r="AH38" s="21" t="n">
         <x:f>O38*AG38+SUM(R38:T38)</x:f>
-        <x:v>150000</x:v>
+        <x:v>105000</x:v>
       </x:c>
       <x:c r="AI38" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ38" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -6483,7 +6483,7 @@
         <x:v>KI-038</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Cam02 v1; Cam12 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
         <x:v>03c</x:v>
@@ -6522,7 +6522,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q39" s="20" t="n">
-        <x:v>70000</x:v>
+        <x:v>55000</x:v>
       </x:c>
       <x:c r="R39" s="20" t="n">
         <x:v>0</x:v>
@@ -6535,13 +6535,13 @@
       </x:c>
       <x:c r="U39" s="21" t="n">
         <x:f>O39*Q39+SUM(R39:T39)</x:f>
-        <x:v>70000</x:v>
+        <x:v>55000</x:v>
       </x:c>
       <x:c r="V39" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W39" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03c</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X39" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -6568,17 +6568,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF39" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>Egyedi ST-01 grafit mellékkocka 300×300×450 mm</x:v>
       </x:c>
       <x:c r="AG39" s="20" t="n">
-        <x:v>70000</x:v>
+        <x:v>55000</x:v>
       </x:c>
       <x:c r="AH39" s="21" t="n">
         <x:f>O39*AG39+SUM(R39:T39)</x:f>
-        <x:v>70000</x:v>
+        <x:v>55000</x:v>
       </x:c>
       <x:c r="AI39" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ39" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -16768,7 +16768,7 @@
         <x:v>KI-123</x:v>
       </x:c>
       <x:c r="D124" s="12" t="str">
-        <x:v>Cam12 v1; Cam03 v2</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E124" s="12" t="str">
         <x:v>11</x:v>
@@ -16807,7 +16807,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q124" s="20" t="n">
-        <x:v>60000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="R124" s="20" t="n">
         <x:v>0</x:v>
@@ -16820,13 +16820,13 @@
       </x:c>
       <x:c r="U124" s="21" t="n">
         <x:f>O124*Q124+SUM(R124:T124)</x:f>
-        <x:v>60000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="V124" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W124" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 11</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X124" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -16853,17 +16853,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF124" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>W02 alapvlies helyett KI-132 textilpanel; kiváltott sor, nincs kettős számolás</x:v>
       </x:c>
       <x:c r="AG124" s="20" t="n">
-        <x:v>60000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AH124" s="21" t="n">
         <x:f>O124*AG124+SUM(R124:T124)</x:f>
-        <x:v>60000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AI124" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ124" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -17857,7 +17857,7 @@
         <x:v>KI-132</x:v>
       </x:c>
       <x:c r="D133" s="12" t="str">
-        <x:v>Cam12 v1; Cam02 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E133" s="12" t="str">
         <x:v>12</x:v>
@@ -17896,7 +17896,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q133" s="20" t="n">
-        <x:v>80000</x:v>
+        <x:v>185000</x:v>
       </x:c>
       <x:c r="R133" s="20" t="n">
         <x:v>0</x:v>
@@ -17909,13 +17909,13 @@
       </x:c>
       <x:c r="U133" s="21" t="n">
         <x:f>O133*Q133+SUM(R133:T133)</x:f>
-        <x:v>80000</x:v>
+        <x:v>185000</x:v>
       </x:c>
       <x:c r="V133" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W133" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 12</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X133" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -17942,17 +17942,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF133" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>W02 2100×2880 mm textilborítású levehető panelmező, nem 150×220 keretelt kép</x:v>
       </x:c>
       <x:c r="AG133" s="20" t="n">
-        <x:v>80000</x:v>
+        <x:v>185000</x:v>
       </x:c>
       <x:c r="AH133" s="21" t="n">
         <x:f>O133*AG133+SUM(R133:T133)</x:f>
-        <x:v>80000</x:v>
+        <x:v>185000</x:v>
       </x:c>
       <x:c r="AI133" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ133" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -17978,7 +17978,7 @@
         <x:v>KI-133</x:v>
       </x:c>
       <x:c r="D134" s="12" t="str">
-        <x:v>Cam12 v1; Cam02 v1</x:v>
+        <x:v>Cam_02/Cam_12 V33_C_v1</x:v>
       </x:c>
       <x:c r="E134" s="12" t="str">
         <x:v>12</x:v>
@@ -18017,7 +18017,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q134" s="20" t="n">
-        <x:v>60000</x:v>
+        <x:v>95000</x:v>
       </x:c>
       <x:c r="R134" s="20" t="n">
         <x:v>0</x:v>
@@ -18030,13 +18030,13 @@
       </x:c>
       <x:c r="U134" s="21" t="n">
         <x:f>O134*Q134+SUM(R134:T134)</x:f>
-        <x:v>60000</x:v>
+        <x:v>95000</x:v>
       </x:c>
       <x:c r="V134" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W134" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 12</x:v>
+        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X134" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -18063,17 +18063,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF134" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>W02 hordozó, hátoldali sínek, rejtett rögzítés; nem képkeret</x:v>
       </x:c>
       <x:c r="AG134" s="20" t="n">
-        <x:v>60000</x:v>
+        <x:v>95000</x:v>
       </x:c>
       <x:c r="AH134" s="21" t="n">
         <x:f>O134*AG134+SUM(R134:T134)</x:f>
-        <x:v>60000</x:v>
+        <x:v>95000</x:v>
       </x:c>
       <x:c r="AI134" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>CP V33 célátvétel: optimalizálás következő csomagban</x:v>
       </x:c>
       <x:c r="AJ134" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -21245,7 +21245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ade8ec045474f4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf2454dfee54dfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21662,15 +21662,15 @@
       </x:c>
       <x:c r="D16" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$E$2:$E$160,A16)</x:f>
-        <x:v>960000</x:v>
+        <x:v>1150000</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$E$2:$E$160,A16)</x:f>
-        <x:v>960000</x:v>
+        <x:v>1150000</x:v>
       </x:c>
       <x:c r="F16" s="18" t="n">
         <x:f>E16-C16</x:f>
-        <x:v>99000</x:v>
+        <x:v>289000</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
         <x:v>W01 teljes panelkompozíció és tusgrafikás torony; W01 alsó négyfrontos médiabútor; W01 rögzítés, szerviznyílás, szerelés; TV készülék 65 col célkategória; Teherhordó TV-konzol; HDMI, hálózat, kábelszervezés, audióigény előirányzat</x:v>
@@ -21714,15 +21714,15 @@
       </x:c>
       <x:c r="D18" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$E$2:$E$160,A18)</x:f>
-        <x:v>220000</x:v>
+        <x:v>160000</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$E$2:$E$160,A18)</x:f>
-        <x:v>220000</x:v>
+        <x:v>160000</x:v>
       </x:c>
       <x:c r="F18" s="18" t="n">
         <x:f>E18-C18</x:f>
-        <x:v>0</x:v>
+        <x:v>-60000</x:v>
       </x:c>
       <x:c r="G18" s="19" t="str">
         <x:v>Grafit dohányzóasztal; Grafit mellékasztal</x:v>
@@ -21974,15 +21974,15 @@
       </x:c>
       <x:c r="D28" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$E$2:$E$160,A28)</x:f>
-        <x:v>465000</x:v>
+        <x:v>405000</x:v>
       </x:c>
       <x:c r="E28" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$E$2:$E$160,A28)</x:f>
-        <x:v>465000</x:v>
+        <x:v>405000</x:v>
       </x:c>
       <x:c r="F28" s="18" t="n">
         <x:f>E28-C28</x:f>
-        <x:v>129000</x:v>
+        <x:v>69000</x:v>
       </x:c>
       <x:c r="G28" s="19" t="str">
         <x:v>W02 papírhatású vlies; W07 folytató tapéta és grafikai vonal; W03 és szemöldök tapéta; W04 tömör mezők tapéta; Alapozó, ragasztó és faljavítás; Tapétázás, sarkok, élek és kapcsolók körbevágása; Szabási és illesztési veszteség; Fejvég feletti és ablak melletti vlies felrakással</x:v>
@@ -22000,15 +22000,15 @@
       </x:c>
       <x:c r="D29" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$160,'Elemregiszter'!$E$2:$E$160,A29)</x:f>
-        <x:v>290000</x:v>
+        <x:v>430000</x:v>
       </x:c>
       <x:c r="E29" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$160,'Elemregiszter'!$E$2:$E$160,A29)</x:f>
-        <x:v>290000</x:v>
+        <x:v>430000</x:v>
       </x:c>
       <x:c r="F29" s="18" t="n">
         <x:f>E29-C29</x:f>
-        <x:v>28000</x:v>
+        <x:v>168000</x:v>
       </x:c>
       <x:c r="G29" s="19" t="str">
         <x:v>W02 eredeti tusgrafika előállítása és nyomdai előkészítése; W02 textilnyomat 150×220 célméret; W02 vékony keret, szállítás és rögzítés; Nappali párnák és takaró; Kerámiák, művészeti könyvek és kisebb növények</x:v>
@@ -22054,15 +22054,15 @@
       </x:c>
       <x:c r="D31" s="18" t="n">
         <x:f>SUM(D2:D30)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
         <x:f>SUM(E2:E30)</x:f>
-        <x:v>20083350</x:v>
+        <x:v>20293350</x:v>
       </x:c>
       <x:c r="F31" s="18" t="n">
         <x:f>SUM(F2:F30)</x:f>
-        <x:v>2472350</x:v>
+        <x:v>2682350</x:v>
       </x:c>
       <x:c r="G31" s="19"/>
     </x:row>

</xml_diff>

<commit_message>
KI-R06: seven current appearance targets, product geometry and artwork proofs, revised costs and conditional drawing handoff
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
@@ -2,29 +2,30 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R2f574edc1084496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="R93808e6a8ddb4ba2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R8c2268fe2a1c4fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R68847b5f72564790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="Rc2ec6f27e02241da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="R83a131b4d086412e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="Rf4e1c924da4547df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="R243504e2e75d459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="Rc44d6faf95294173"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="Rd5abdde4f7cb40a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="Rcdaeb870fc5b4eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="Rd3f9bcf825194138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="Rbd416981ed3245ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="Rc8062f7e037b426f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="R7392b12a77c9407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R53a4e4d0014541e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="Rf89ed3fefb1a4e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="Rf027cb6252fd44df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="R67b1a1fe16184604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="Rbbf63d81d4dd427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R9dbc81a4226a47ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R4102b6bf46f744be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="R828f89c339d34e93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R36f923b2bd5c428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="R5a663db2597c42b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R6a5dbed989eb4e2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R00bc4a9d73304419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="Re2eddac4a63c4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="Rad3f698ce8b344e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="R247f37bcf5b84807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="R788bc37c0d80435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="R918c68f7a6924c54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="R33b845d9132045c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="R66fe7959d04545b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="Rc87a2cb0bbaa418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="Ra2d833928f994d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="R916d3c7ce21648d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="R90cba8e611bb4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R2c972e89bad4460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="Recea1fd0f1f8420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="R62314806f80b4a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="Rd089dc3f38fd44f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="R9ce53e5c38804796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R7744d4f00a18492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R11c0036e45f64e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="Rcd609916148c4f66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 változások" sheetId="24" r:id="Refa2a637b72244b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +101,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -110,6 +111,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF303E3C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF303C3B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -185,7 +191,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="62">
+  <x:cellXfs count="64">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -351,6 +357,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3148,11 +3160,11 @@
       </x:c>
       <x:c r="D44" s="19" t="n">
         <x:f>'Elemregiszter'!U44</x:f>
-        <x:v>189900</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="E44" s="19" t="n">
         <x:f>D44-C44</x:f>
-        <x:v>0</x:v>
+        <x:v>60100</x:v>
       </x:c>
       <x:c r="F44" s="19" t="str">
         <x:v>Matrac külön; fióknyitás, éjjeli ütközés, 202cm külső hossz ellenőrzése.</x:v>
@@ -3170,11 +3182,11 @@
       </x:c>
       <x:c r="D45" s="19" t="n">
         <x:f>'Elemregiszter'!U45</x:f>
-        <x:v>260000</x:v>
+        <x:v>229900</x:v>
       </x:c>
       <x:c r="E45" s="19" t="n">
         <x:f>D45-C45</x:f>
-        <x:v>0</x:v>
+        <x:v>-30100</x:v>
       </x:c>
       <x:c r="F45" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -3324,11 +3336,11 @@
       </x:c>
       <x:c r="D52" s="19" t="n">
         <x:f>'Elemregiszter'!U52</x:f>
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="E52" s="19" t="n">
         <x:f>D52-C52</x:f>
-        <x:v>120000</x:v>
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="F52" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -4776,11 +4788,11 @@
       </x:c>
       <x:c r="D118" s="19" t="n">
         <x:f>'Elemregiszter'!U118</x:f>
-        <x:v>35980</x:v>
+        <x:v>45980</x:v>
       </x:c>
       <x:c r="E118" s="19" t="n">
         <x:f>D118-C118</x:f>
-        <x:v>-34020</x:v>
+        <x:v>-24020</x:v>
       </x:c>
       <x:c r="F118" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -19679,11 +19691,11 @@
         <x:v>Fő előrejelzés</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:f>SUM('Elemregiszter'!U2:U175)</x:f>
-        <x:v>23912890</x:v>
+        <x:f>SUM('Elemregiszter'!U2:U178)</x:f>
+        <x:v>24482890</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>R05: teljes R04 bútorváltozat + teljes W02 + biciklitartó. Árazási munkaváltozat, nem rendelési jóváhagyás.</x:v>
+        <x:v>R06: hét új célkép; pontos termékformák, grafikapróbák, magas gardróbfrontok és T07 kiegészítések. Nem rendelési engedély.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -19691,11 +19703,11 @@
         <x:v>Gazdaságos javaslat</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:f>SUM('Elemregiszter'!AH2:AH175)</x:f>
-        <x:v>23659890</x:v>
+        <x:f>SUM('Elemregiszter'!AH2:AH178)</x:f>
+        <x:v>24229890</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>Azonos tárolókapacitás. Síkabb W01, vlies W02, fix fürdődugalj; mindhárom változtatás döntésre és ajánlatra vár.</x:v>
+        <x:v>Összehasonlítható takarékos változat:253000Ft dokumentált megtakarítás;18M továbbra sem igazolt.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -19704,7 +19716,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>B7-B5</x:f>
-        <x:v>5912890</x:v>
+        <x:v>6482890</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19716,7 +19728,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>B8-B5</x:f>
-        <x:v>5659890</x:v>
+        <x:v>6229890</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19727,8 +19739,8 @@
         <x:v>Ellenőrzött webshopár rész</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U175,'Elemregiszter'!V2:V175,"ellenőrzött webshopár")</x:f>
-        <x:v>2332340</x:v>
+        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!V2:V178,"ellenőrzött webshopár")</x:f>
+        <x:v>2142440</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
         <x:v>Termékérték; szállítás/szerelés becslése külön maradhat</x:v>
@@ -19739,7 +19751,7 @@
         <x:v>Beszállítói ajánlat rész</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U175,'Elemregiszter'!V2:V175,"beszállítói ajánlat")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!V2:V178,"beszállítói ajánlat")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
@@ -19752,7 +19764,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>B7-B11-B12</x:f>
-        <x:v>21580550</x:v>
+        <x:v>22340450</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>Minden nem igazolt ár</x:v>
@@ -19763,7 +19775,7 @@
         <x:v>Megrendelt érték</x:v>
       </x:c>
       <x:c r="B14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U175,'Elemregiszter'!AC2:AC175,"megrendelt")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!AC2:AC178,"megrendelt")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
@@ -19775,11 +19787,11 @@
         <x:v>Tételszám</x:v>
       </x:c>
       <x:c r="B15" s="18" t="n">
-        <x:f>COUNTA('Elemregiszter'!C2:C175)</x:f>
-        <x:v>174</x:v>
+        <x:f>COUNTA('Elemregiszter'!C2:C178)</x:f>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>174 élő költségsor; R05 anyag és kapacitás kiegészítéssel.</x:v>
+        <x:v>177 költségsor; a külön2M tartalékból0Ft felhasználva.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -19835,11 +19847,11 @@
         <x:v>teljes lakás</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A22)</x:f>
         <x:v>1953790</x:v>
       </x:c>
       <x:c r="C22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A22)</x:f>
         <x:v>1953790</x:v>
       </x:c>
     </x:row>
@@ -19848,11 +19860,11 @@
         <x:v>02</x:v>
       </x:c>
       <x:c r="B23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A23)</x:f>
         <x:v>3287990</x:v>
       </x:c>
       <x:c r="C23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A23)</x:f>
         <x:v>3287990</x:v>
       </x:c>
     </x:row>
@@ -19861,11 +19873,11 @@
         <x:v>03</x:v>
       </x:c>
       <x:c r="B24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A24)</x:f>
         <x:v>971070</x:v>
       </x:c>
       <x:c r="C24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A24)</x:f>
         <x:v>971070</x:v>
       </x:c>
     </x:row>
@@ -19874,11 +19886,11 @@
         <x:v>04</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A25)</x:f>
         <x:v>3742190</x:v>
       </x:c>
       <x:c r="C25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A25)</x:f>
         <x:v>3594190</x:v>
       </x:c>
     </x:row>
@@ -19887,12 +19899,12 @@
         <x:v>05.1</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A26)</x:f>
-        <x:v>3685500</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A26)</x:f>
+        <x:v>3805500</x:v>
       </x:c>
       <x:c r="C26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A26)</x:f>
-        <x:v>3685500</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A26)</x:f>
+        <x:v>3805500</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
@@ -19900,11 +19912,11 @@
         <x:v>05.2</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A27)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="C27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A27)</x:f>
         <x:v>1179980</x:v>
       </x:c>
     </x:row>
@@ -19913,11 +19925,11 @@
         <x:v>05.3</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A28)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="C28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A28)</x:f>
         <x:v>1157380</x:v>
       </x:c>
     </x:row>
@@ -19926,11 +19938,11 @@
         <x:v>01</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A29)</x:f>
         <x:v>440000</x:v>
       </x:c>
       <x:c r="C29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A29)</x:f>
         <x:v>440000</x:v>
       </x:c>
     </x:row>
@@ -19939,11 +19951,11 @@
         <x:v>07</x:v>
       </x:c>
       <x:c r="B30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A30)</x:f>
         <x:v>40000</x:v>
       </x:c>
       <x:c r="C30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A30)</x:f>
         <x:v>40000</x:v>
       </x:c>
     </x:row>
@@ -19952,11 +19964,11 @@
         <x:v>06.1 / elhelyezés PENDING</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A31)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A31)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="C31" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A31)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A31)</x:f>
         <x:v>485000</x:v>
       </x:c>
     </x:row>
@@ -19965,12 +19977,12 @@
         <x:v>06.2</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A32)</x:f>
-        <x:v>935000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A32)</x:f>
+        <x:v>1385000</x:v>
       </x:c>
       <x:c r="C32" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A32)</x:f>
-        <x:v>830000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A32)</x:f>
+        <x:v>1280000</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
@@ -19978,11 +19990,11 @@
         <x:v>06.1</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A33)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A33)</x:f>
         <x:v>255000</x:v>
       </x:c>
       <x:c r="C33" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A33)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A33)</x:f>
         <x:v>255000</x:v>
       </x:c>
     </x:row>
@@ -19991,11 +20003,11 @@
         <x:v>08</x:v>
       </x:c>
       <x:c r="B34" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A34)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A34)</x:f>
         <x:v>75000</x:v>
       </x:c>
       <x:c r="C34" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A34)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A34)</x:f>
         <x:v>75000</x:v>
       </x:c>
     </x:row>
@@ -20004,11 +20016,11 @@
         <x:v>06.1 / 06.2 / 08</x:v>
       </x:c>
       <x:c r="B35" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A35)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A35)</x:f>
         <x:v>35000</x:v>
       </x:c>
       <x:c r="C35" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A35)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A35)</x:f>
         <x:v>35000</x:v>
       </x:c>
     </x:row>
@@ -20017,11 +20029,11 @@
         <x:v>01 / 07 / 08</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A36)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A36)</x:f>
         <x:v>130000</x:v>
       </x:c>
       <x:c r="C36" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A36)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A36)</x:f>
         <x:v>130000</x:v>
       </x:c>
     </x:row>
@@ -20030,11 +20042,11 @@
         <x:v>06.1 / 06.2</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A37)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A37)</x:f>
         <x:v>340000</x:v>
       </x:c>
       <x:c r="C37" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A37)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A37)</x:f>
         <x:v>340000</x:v>
       </x:c>
     </x:row>
@@ -20043,11 +20055,11 @@
         <x:v>04 / 07</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A38)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A38)</x:f>
         <x:v>315000</x:v>
       </x:c>
       <x:c r="C38" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A38)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A38)</x:f>
         <x:v>315000</x:v>
       </x:c>
     </x:row>
@@ -20056,11 +20068,11 @@
         <x:v>09 terasz Ny</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A39)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A39)</x:f>
         <x:v>2000000</x:v>
       </x:c>
       <x:c r="C39" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A39)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A39)</x:f>
         <x:v>2000000</x:v>
       </x:c>
     </x:row>
@@ -20069,11 +20081,11 @@
         <x:v>10 terasz K</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A40)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A40)</x:f>
         <x:v>1150000</x:v>
       </x:c>
       <x:c r="C40" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A40)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A40)</x:f>
         <x:v>1150000</x:v>
       </x:c>
     </x:row>
@@ -20082,11 +20094,11 @@
         <x:v>09 / 10 / 11 / 12 / 13 kültér</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A41)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A41)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="C41" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A41)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A41)</x:f>
         <x:v>590000</x:v>
       </x:c>
     </x:row>
@@ -20095,11 +20107,11 @@
         <x:v>01 / 04</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A42)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A42)</x:f>
         <x:v>360000</x:v>
       </x:c>
       <x:c r="C42" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$B$2:$B$175,A42)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A42)</x:f>
         <x:v>360000</x:v>
       </x:c>
     </x:row>
@@ -20129,11 +20141,11 @@
         <x:v>Tervezés</x:v>
       </x:c>
       <x:c r="B46" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A46)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A46)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="C46" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A46)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A46)</x:f>
         <x:v>420000</x:v>
       </x:c>
     </x:row>
@@ -20142,12 +20154,12 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="B47" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A47)</x:f>
-        <x:v>6136000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A47)</x:f>
+        <x:v>6216000</x:v>
       </x:c>
       <x:c r="C47" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A47)</x:f>
-        <x:v>6036000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A47)</x:f>
+        <x:v>6116000</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="30" customHeight="1">
@@ -20155,11 +20167,11 @@
         <x:v>Gépek</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A48)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A48)</x:f>
         <x:v>1770000</x:v>
       </x:c>
       <x:c r="C48" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A48)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A48)</x:f>
         <x:v>1770000</x:v>
       </x:c>
     </x:row>
@@ -20168,11 +20180,11 @@
         <x:v>Vízszerelés</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A49)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A49)</x:f>
         <x:v>412990</x:v>
       </x:c>
       <x:c r="C49" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A49)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A49)</x:f>
         <x:v>412990</x:v>
       </x:c>
     </x:row>
@@ -20181,12 +20193,12 @@
         <x:v>Bútor</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A50)</x:f>
-        <x:v>4898330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A50)</x:f>
+        <x:v>4928330</x:v>
       </x:c>
       <x:c r="C50" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A50)</x:f>
-        <x:v>4898330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A50)</x:f>
+        <x:v>4928330</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="30" customHeight="1">
@@ -20194,11 +20206,11 @@
         <x:v>Elektronika</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A51)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A51)</x:f>
         <x:v>680000</x:v>
       </x:c>
       <x:c r="C51" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A51)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A51)</x:f>
         <x:v>680000</x:v>
       </x:c>
     </x:row>
@@ -20207,11 +20219,11 @@
         <x:v>Textil</x:v>
       </x:c>
       <x:c r="B52" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A52)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A52)</x:f>
         <x:v>1330000</x:v>
       </x:c>
       <x:c r="C52" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A52)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A52)</x:f>
         <x:v>1330000</x:v>
       </x:c>
     </x:row>
@@ -20220,11 +20232,11 @@
         <x:v>Művészet</x:v>
       </x:c>
       <x:c r="B53" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A53)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A53)</x:f>
         <x:v>611000</x:v>
       </x:c>
       <x:c r="C53" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A53)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A53)</x:f>
         <x:v>563000</x:v>
       </x:c>
     </x:row>
@@ -20233,12 +20245,12 @@
         <x:v>Villamos</x:v>
       </x:c>
       <x:c r="B54" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A54)</x:f>
-        <x:v>2190360</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A54)</x:f>
+        <x:v>2200360</x:v>
       </x:c>
       <x:c r="C54" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A54)</x:f>
-        <x:v>2190360</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A54)</x:f>
+        <x:v>2200360</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="30" customHeight="1">
@@ -20246,11 +20258,11 @@
         <x:v>Üveges</x:v>
       </x:c>
       <x:c r="B55" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A55)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A55)</x:f>
         <x:v>180000</x:v>
       </x:c>
       <x:c r="C55" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A55)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A55)</x:f>
         <x:v>180000</x:v>
       </x:c>
     </x:row>
@@ -20259,11 +20271,11 @@
         <x:v>Kiegészítők</x:v>
       </x:c>
       <x:c r="B56" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A56)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A56)</x:f>
         <x:v>250000</x:v>
       </x:c>
       <x:c r="C56" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A56)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A56)</x:f>
         <x:v>250000</x:v>
       </x:c>
     </x:row>
@@ -20272,11 +20284,11 @@
         <x:v>Falfelület</x:v>
       </x:c>
       <x:c r="B57" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A57)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A57)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="C57" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A57)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A57)</x:f>
         <x:v>405000</x:v>
       </x:c>
     </x:row>
@@ -20285,11 +20297,11 @@
         <x:v>Kert és terasz</x:v>
       </x:c>
       <x:c r="B58" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A58)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A58)</x:f>
         <x:v>2590000</x:v>
       </x:c>
       <x:c r="C58" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A58)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A58)</x:f>
         <x:v>2590000</x:v>
       </x:c>
     </x:row>
@@ -20298,11 +20310,11 @@
         <x:v>Logisztika</x:v>
       </x:c>
       <x:c r="B59" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$G$2:$G$175,A59)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A59)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="C59" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$G$2:$G$175,A59)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A59)</x:f>
         <x:v>510000</x:v>
       </x:c>
     </x:row>
@@ -20332,11 +20344,11 @@
         <x:v>FIX</x:v>
       </x:c>
       <x:c r="B63" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$F$2:$F$175,A63)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$F$2:$F$178,A63)</x:f>
         <x:v>9510350</x:v>
       </x:c>
       <x:c r="C63" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$F$2:$F$175,A63)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$F$2:$F$178,A63)</x:f>
         <x:v>9510350</x:v>
       </x:c>
     </x:row>
@@ -20345,12 +20357,12 @@
         <x:v>STÍLUS</x:v>
       </x:c>
       <x:c r="B64" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$F$2:$F$175,A64)</x:f>
-        <x:v>12873330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$F$2:$F$178,A64)</x:f>
+        <x:v>12993330</x:v>
       </x:c>
       <x:c r="C64" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$F$2:$F$175,A64)</x:f>
-        <x:v>12725330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$F$2:$F$178,A64)</x:f>
+        <x:v>12845330</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="30" customHeight="1">
@@ -20379,12 +20391,12 @@
         <x:v>nem megrendelt</x:v>
       </x:c>
       <x:c r="B68" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$AC$2:$AC$175,A68)</x:f>
-        <x:v>22383680</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$AC$2:$AC$178,A68)</x:f>
+        <x:v>22503680</x:v>
       </x:c>
       <x:c r="C68" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$AC$2:$AC$175,A68)</x:f>
-        <x:v>22235680</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$AC$2:$AC$178,A68)</x:f>
+        <x:v>22355680</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -20415,8 +20427,8 @@
         <x:v>Alsó sáv</x:v>
       </x:c>
       <x:c r="B74" s="30" t="n">
-        <x:f>SUM('Elemregiszter'!BA2:BA175)</x:f>
-        <x:v>20414580</x:v>
+        <x:f>SUM('Elemregiszter'!BA2:BA178)</x:f>
+        <x:v>20841595</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>Sorok alsó feltételezéseinek összege</x:v>
@@ -20427,8 +20439,8 @@
         <x:v>Felső sáv</x:v>
       </x:c>
       <x:c r="B75" s="30" t="n">
-        <x:f>SUM('Elemregiszter'!BB2:BB175)</x:f>
-        <x:v>32032116</x:v>
+        <x:f>SUM('Elemregiszter'!BB2:BB178)</x:f>
+        <x:v>32952998</x:v>
       </x:c>
       <x:c r="C75" t="str">
         <x:v>Sorok felső feltételezéseinek összege</x:v>
@@ -20473,7 +20485,7 @@
         <x:v>AT8-01</x:v>
       </x:c>
       <x:c r="B80" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A80)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A80)</x:f>
         <x:v>380990</x:v>
       </x:c>
       <x:c r="C80" t="str">
@@ -20485,7 +20497,7 @@
         <x:v>T-0-26</x:v>
       </x:c>
       <x:c r="B81" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A81)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A81)</x:f>
         <x:v>165000</x:v>
       </x:c>
       <x:c r="C81" t="str">
@@ -20497,7 +20509,7 @@
         <x:v>AT8-01 / T-0-26</x:v>
       </x:c>
       <x:c r="B82" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$B$2:$B$175,A82)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A82)</x:f>
         <x:v>174000</x:v>
       </x:c>
       <x:c r="C82" t="str">
@@ -20509,7 +20521,7 @@
         <x:v>Fagyasztó és kapcsolódó munka</x:v>
       </x:c>
       <x:c r="B83" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$C$2:$C$175,"KI-CP3-F01")+SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$C$2:$C$175,"KI-CP3-F02")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$C$2:$C$178,"KI-CP3-F01")+SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$C$2:$C$178,"KI-CP3-F02")</x:f>
         <x:v>334990</x:v>
       </x:c>
       <x:c r="C83" t="str">
@@ -20522,7 +20534,7 @@
       </x:c>
       <x:c r="B84" s="30" t="n">
         <x:f>B7-B83</x:f>
-        <x:v>23577900</x:v>
+        <x:v>24147900</x:v>
       </x:c>
       <x:c r="C84" t="str">
         <x:v>Nem automatikusan kiválasztott megtakarítás</x:v>
@@ -24057,15 +24069,15 @@
       </x:c>
       <x:c r="C5" s="55" t="n">
         <x:f>'Elemregiszter'!U52</x:f>
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="D5" s="55" t="n">
         <x:f>C5-B5</x:f>
-        <x:v>120000</x:v>
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="E5" s="55" t="n">
         <x:f>'Elemregiszter'!AH52</x:f>
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="F5" s="55" t="n">
         <x:f>C5-E5</x:f>
@@ -26713,6 +26725,324 @@
       </x:c>
       <x:c r="O41" s="19" t="str">
         <x:v>Tervi kapacitás, nem felmért vagy garantált tárgybeférés.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="105" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="70" customHeight="1">
+      <x:c r="A1" s="63" t="str">
+        <x:v>Elem</x:v>
+      </x:c>
+      <x:c r="B1" s="63" t="str">
+        <x:v>R05 Ft</x:v>
+      </x:c>
+      <x:c r="C1" s="63" t="str">
+        <x:v>R06 Ft</x:v>
+      </x:c>
+      <x:c r="D1" s="63" t="str">
+        <x:v>Eltérés Ft</x:v>
+      </x:c>
+      <x:c r="E1" s="63" t="str">
+        <x:v>Műszaki változás</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="70" customHeight="1">
+      <x:c r="A2" s="1" t="str">
+        <x:v>KI-044</x:v>
+      </x:c>
+      <x:c r="B2" s="29" t="n">
+        <x:v>260000</x:v>
+      </x:c>
+      <x:c r="C2" s="29" t="n">
+        <x:f>'Elemregiszter'!U45</x:f>
+        <x:v>229900</x:v>
+      </x:c>
+      <x:c r="D2" s="29" t="n">
+        <x:f>C2-B2</x:f>
+        <x:v>-30100</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>VÅGSTRANDA pontos méret és friss ár, -30100 Ft; keménység kipróbálandó.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="70" customHeight="1">
+      <x:c r="A3" s="1" t="str">
+        <x:v>KI-117</x:v>
+      </x:c>
+      <x:c r="B3" s="29" t="n">
+        <x:v>35980</x:v>
+      </x:c>
+      <x:c r="C3" s="29" t="n">
+        <x:f>'Elemregiszter'!U118</x:f>
+        <x:v>45980</x:v>
+      </x:c>
+      <x:c r="D3" s="29" t="n">
+        <x:f>C3-B3</x:f>
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>FADO25cm helyett20cm Rondo; +10000Ft. Összetett csomag, nem teljes fix ajánlat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="70" customHeight="1">
+      <x:c r="A4" s="1" t="str">
+        <x:v>KI-043</x:v>
+      </x:c>
+      <x:c r="B4" s="29" t="n">
+        <x:v>189900</x:v>
+      </x:c>
+      <x:c r="C4" s="29" t="n">
+        <x:f>'Elemregiszter'!U44</x:f>
+        <x:v>250000</x:v>
+      </x:c>
+      <x:c r="D4" s="29" t="n">
+        <x:f>C4-B4</x:f>
+        <x:v>60100</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>NORDLI oldalfiókok helyett felnyíló tároló: éjjelikkel való használati ütközés csökkentése. +60100Ft becslés.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="70" customHeight="1">
+      <x:c r="A5" s="1" t="str">
+        <x:v>KI-051</x:v>
+      </x:c>
+      <x:c r="B5" s="29" t="n">
+        <x:v>370000</x:v>
+      </x:c>
+      <x:c r="C5" s="29" t="n">
+        <x:f>'Elemregiszter'!U52</x:f>
+        <x:v>450000</x:v>
+      </x:c>
+      <x:c r="D5" s="29" t="n">
+        <x:f>C5-B5</x:f>
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>Déli vízszintes frontosztás elhagyva a T05 alapján; belső kapacitás megmarad. +80000Ft előirányzat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="1" t="str">
+        <x:v>KI-011</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="n">
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="C6" s="29" t="n">
+        <x:f>'Elemregiszter'!U12</x:f>
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="D6" s="29" t="n">
+        <x:f>C6-B6</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>F274 beton helyett F243 finom erezetű kődekor.150000Ft csomagkeret nem változik; széles lapra külön ajánlat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="70" customHeight="1">
+      <x:c r="A7" s="1" t="str">
+        <x:v>KI-012</x:v>
+      </x:c>
+      <x:c r="B7" s="29" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="C7" s="29" t="n">
+        <x:f>'Elemregiszter'!U13</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="D7" s="29" t="n">
+        <x:f>C7-B7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Konyha minden nézetében egységes kődekor; költség változatlan.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="70" customHeight="1">
+      <x:c r="A8" s="1" t="str">
+        <x:v>KI-036</x:v>
+      </x:c>
+      <x:c r="B8" s="29" t="n">
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="C8" s="29" t="n">
+        <x:f>'Elemregiszter'!U37</x:f>
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="D8" s="29" t="n">
+        <x:f>C8-B8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Pontos SKU megerősítve; új méretezett forma a régi dobozproxy helyett.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="70" customHeight="1">
+      <x:c r="A9" s="1" t="str">
+        <x:v>KI-028</x:v>
+      </x:c>
+      <x:c r="B9" s="29" t="n">
+        <x:v>259990</x:v>
+      </x:c>
+      <x:c r="C9" s="29" t="n">
+        <x:f>'Elemregiszter'!U29</x:f>
+        <x:v>259990</x:v>
+      </x:c>
+      <x:c r="D9" s="29" t="n">
+        <x:f>C9-B9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Valódi lábszerkezetet mutató modell.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="70" customHeight="1">
+      <x:c r="A10" s="1" t="str">
+        <x:v>KI-029</x:v>
+      </x:c>
+      <x:c r="B10" s="29" t="n">
+        <x:v>451080</x:v>
+      </x:c>
+      <x:c r="C10" s="29" t="n">
+        <x:f>'Elemregiszter'!U30</x:f>
+        <x:v>451080</x:v>
+      </x:c>
+      <x:c r="D10" s="29" t="n">
+        <x:f>C10-B10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>Hajlított kőris háttámla, világosszürke zsenília és fekete acélláb a képeken is.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="70" customHeight="1">
+      <x:c r="A11" s="1" t="str">
+        <x:v>KI-109</x:v>
+      </x:c>
+      <x:c r="B11" s="29" t="n">
+        <x:v>260000</x:v>
+      </x:c>
+      <x:c r="C11" s="29" t="n">
+        <x:f>'Elemregiszter'!U110</x:f>
+        <x:v>260000</x:v>
+      </x:c>
+      <x:c r="D11" s="29" t="n">
+        <x:f>C11-B11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="1" t="str">
+        <x:v>A tényleges760mm Somar forma követése.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="70" customHeight="1">
+      <x:c r="A12" s="1" t="str">
+        <x:v>KI-076</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="C12" s="29" t="n">
+        <x:f>'Elemregiszter'!U77</x:f>
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="D12" s="29" t="n">
+        <x:f>C12-B12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="1" t="str">
+        <x:v>Vendégszobai éjjeli a munkaszék kihúzási sávjából az ágy fejrészéhez kerül.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="70" customHeight="1">
+      <x:c r="A13" s="1" t="str">
+        <x:v>KI-091</x:v>
+      </x:c>
+      <x:c r="B13" s="29" t="n">
+        <x:v>180000</x:v>
+      </x:c>
+      <x:c r="C13" s="29" t="n">
+        <x:f>'Elemregiszter'!U92</x:f>
+        <x:v>180000</x:v>
+      </x:c>
+      <x:c r="D13" s="29" t="n">
+        <x:f>C13-B13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="str">
+        <x:v>Az örökölt, zuhanytálcán keresztbe álló üveg helyett a tálca éléhez igazított tervváltozat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="70" customHeight="1">
+      <x:c r="A14" s="1" t="str">
+        <x:v>KI-R06-01</x:v>
+      </x:c>
+      <x:c r="B14" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="29" t="n">
+        <x:f>'Elemregiszter'!U176</x:f>
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="D14" s="29" t="n">
+        <x:f>C14-B14</x:f>
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="str">
+        <x:v>900×200×1400mm; z1300;600ajtó+300nyitottfülke. Korpusz45000+front/lamella65000+vasalat20000+LED/táp25000+szerelés65000.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="1" t="str">
+        <x:v>KI-R06-02</x:v>
+      </x:c>
+      <x:c r="B15" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="29" t="n">
+        <x:f>'Elemregiszter'!U177</x:f>
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="D15" s="29" t="n">
+        <x:f>C15-B15</x:f>
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="str">
+        <x:v>900×2400mm tervi felület; 2.16m²+15%rendelési ráhagyás. Védett hátoldali nyomat, üveg/szakági rendszer50000+grafika/nyomat25000+rögzítés35000. Zuhanyzónában akasztó/pad nem kerülhet elé.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="1" t="str">
+        <x:v>KI-R06-03</x:v>
+      </x:c>
+      <x:c r="B16" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="29" t="n">
+        <x:f>'Elemregiszter'!U178</x:f>
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="D16" s="29" t="n">
+        <x:f>C16-B16</x:f>
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="str">
+        <x:v>400×1200mm tervi befoglaló; késztermék70000+bekötés/rögzítés50000. Pontos modell, hőigény, zóna és kiállás nyitott; meglévő esetén csak igazolás után levonható.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28653,19 +28983,19 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>EGGER F243 ST76 / 4100×920×38</x:v>
       </x:c>
       <x:c r="K12" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>https://www.okftfaaruhaz.hu/ML-EGGER-F243-ST76-4100x600x38mm-munkalap</x:v>
       </x:c>
       <x:c r="L12" s="19" t="str">
-        <x:v>K-08: 1460×620×38 mm; K-09: 1600×620×38 mm</x:v>
+        <x:v>1460×620 +1600×620 +900×620; 4100×920 nyerslapból</x:v>
       </x:c>
       <x:c r="M12" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N12" s="19" t="str">
-        <x:v>MAT-07</x:v>
+        <x:v>Világosszürke Candela márvány dekor, laminált forgácslap; nem valódi kő</x:v>
       </x:c>
       <x:c r="O12" s="19" t="n">
         <x:v>1</x:v>
@@ -28693,7 +29023,7 @@
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W12" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 02a</x:v>
+        <x:v>96750Ft széles lap jelzett kereskedői ár +53250Ft szabás/él/kivágás előirányzat; széles SKU véglegesítendő</x:v>
       </x:c>
       <x:c r="X12" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -28705,7 +29035,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="AA12" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>Képi kőhatás közelítése lamináttal; élek és ismétlődés látszhat. 600mm lap NEM elegendő620mm mélységre.</x:v>
       </x:c>
       <x:c r="AB12" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -28821,7 +29151,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J13" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>EGGER F243 ST76 hátfal</x:v>
       </x:c>
       <x:c r="K13" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -28861,7 +29191,7 @@
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W13" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 02a</x:v>
+        <x:v>4100×640×8 jelzett59445Ft +40555Ft szabás/ragasztás/él előirányzat. Nem dupla munkadíj a KI-014-gyel; ajánlatban bontandó</x:v>
       </x:c>
       <x:c r="X13" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -28873,7 +29203,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="AA13" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>Azonos dekor az összes konyhanézetben; mosható hátfal, főzőlap gyártói távolságával</x:v>
       </x:c>
       <x:c r="AB13" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -31549,10 +31879,10 @@
         <x:v>ellenőrzött webshopár</x:v>
       </x:c>
       <x:c r="W29" s="19" t="str">
-        <x:v>https://www.westwing.hu/toni-ovalis-alaku-fa-etkezoasztal-200-x-90-cm-hu-19wes60483.html?simple=DEQ19WES60483-225182</x:v>
+        <x:v>Westwing HU SKU160cm259990Ft</x:v>
       </x:c>
       <x:c r="X29" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="Y29" s="19" t="str">
         <x:v>9–11 munkanap; feláras szállítás; 10 év gyártói garancia</x:v>
@@ -31561,7 +31891,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="AA29" s="19" t="str">
-        <x:v>Az URL 200 cm-et tartalmaz, de a kiválasztott SKU 160-as. A render hosszabb asztalbenyomása nem írja felül a 160-as befoglalót.</x:v>
+        <x:v>160×90 ovális tölgy asztal, két hajlított laplábbal; nem a renderben esetenként megjelenő központi tömb.</x:v>
       </x:c>
       <x:c r="AB29" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -31607,7 +31937,7 @@
         <x:v>drawings/P-01_alaprajz.pdf</x:v>
       </x:c>
       <x:c r="AP29" s="1" t="str">
-        <x:v>KI_KI-028; KI_KI-028_base</x:v>
+        <x:v>R06_Toni*</x:v>
       </x:c>
       <x:c r="AQ29" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
@@ -31775,13 +32105,13 @@
         <x:v>drawings/P-01_alaprajz.pdf</x:v>
       </x:c>
       <x:c r="AP30" s="1" t="str">
-        <x:v>KI_KI-029-1; KI_KI-029-2; KI_KI-029-3; KI_KI-029-4; KI_KI-029-5; KI_KI-029-6</x:v>
+        <x:v>R06_Eamy_*</x:v>
       </x:c>
       <x:c r="AQ30" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
       </x:c>
       <x:c r="AR30" s="1" t="str">
-        <x:v>felmérés/gyártói rajz szükséges</x:v>
+        <x:v>Gyártói55×53×75cm, ülés46cm; fotó alapján görbített háttámla rekonstrukció</x:v>
       </x:c>
       <x:c r="AS30" s="1" t="str">
         <x:v>HUF</x:v>
@@ -32893,10 +33223,10 @@
         <x:v>ellenőrzött webshopár</x:v>
       </x:c>
       <x:c r="W37" s="19" t="str">
-        <x:v>https://www.westwing.hu/lennon-modularis-sarokkanape-hu-21wes12329.html?simple=DEQ21WES12329-168260</x:v>
+        <x:v>Westwing HU pontos SKU JSON-LD:800000Ft; HU szállítás visszaigazolása nincs</x:v>
       </x:c>
       <x:c r="X37" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="Y37" s="19" t="str">
         <x:v>8–9 hét; szállítás feláras; 10 év gyártói garancia az oldalon</x:v>
@@ -32905,7 +33235,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="AA37" s="19" t="str">
-        <x:v>A prompt főhorgonya; a render lágyabb párnatagolását és taupe tónusát nem tekintjük gyári pontosságúnak. A jobb L irány a termékfotó szerinti, helyiségbe forgatva ellenőrizendő.</x:v>
+        <x:v>Alacsony, széles karú jobb sarokkanapé; a célkép szövete és párnázottsága eltérhet.</x:v>
       </x:c>
       <x:c r="AB37" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -32951,13 +33281,13 @@
         <x:v>drawings/P-01_alaprajz.pdf</x:v>
       </x:c>
       <x:c r="AP37" s="1" t="str">
-        <x:v>KI_KI-036_backrun; KI_KI-036_chaise</x:v>
+        <x:v>R06_Lennon_*</x:v>
       </x:c>
       <x:c r="AQ37" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
       </x:c>
       <x:c r="AR37" s="1" t="str">
-        <x:v>felmérés/gyártói rajz szükséges</x:v>
+        <x:v>Gyártói2380×1800×680; fotó/méret alapján felépített forma, nem gyári3D</x:v>
       </x:c>
       <x:c r="AS37" s="1" t="str">
         <x:v>HUF</x:v>
@@ -34023,19 +34353,19 @@
         <x:v>Bútor</x:v>
       </x:c>
       <x:c r="H44" s="19" t="str">
-        <x:v>180×200 ágykeret és tartóalap</x:v>
+        <x:v>BED-01 egyedi kárpitozott tárolóágy, közös felnyíló kerettel</x:v>
       </x:c>
       <x:c r="I44" s="19" t="str">
-        <x:v>IKEA</x:v>
+        <x:v>Egyedi ajánlatkérés</x:v>
       </x:c>
       <x:c r="J44" s="19" t="str">
-        <x:v>203.498.53</x:v>
+        <x:v>BED-01-R06</x:v>
       </x:c>
       <x:c r="K44" s="19" t="str">
         <x:v>https://www.ikea.com/hu/hu/p/nordli-agykeret-taroloval-feher-20349853/</x:v>
       </x:c>
       <x:c r="L44" s="19" t="str">
-        <x:v>külső180×202×30</x:v>
+        <x:v>2020×1800×300 mm külső, matrac1800×2000</x:v>
       </x:c>
       <x:c r="M44" s="19" t="str">
         <x:v>fehér</x:v>
@@ -34050,7 +34380,7 @@
         <x:v>db</x:v>
       </x:c>
       <x:c r="Q44" s="20" t="n">
-        <x:v>189900</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="R44" s="20" t="n">
         <x:v>0</x:v>
@@ -34063,13 +34393,13 @@
       </x:c>
       <x:c r="U44" s="21" t="n">
         <x:f>O44*Q44+SUM(R44:T44)</x:f>
-        <x:v>189900</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="V44" s="19" t="str">
-        <x:v>ellenőrzött webshopár</x:v>
+        <x:v>Becslés</x:v>
       </x:c>
       <x:c r="W44" s="19" t="str">
-        <x:v>https://www.ikea.com/hu/hu/p/nordli-agykeret-taroloval-feher-20349853/</x:v>
+        <x:v>R06 bontás: váz80000+kárpit50000+közös keret és kétoldali emelőszerkezet80000+összeépítés40000; vasalat ajánlatra vár</x:v>
       </x:c>
       <x:c r="X44" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -34081,7 +34411,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="AA44" s="19" t="str">
-        <x:v>A fehér fiókos doboz nem a render puha, szürke ágyoldala. Egyedi fejvég külön; esetleges kárpitborítás nem része az árnak és nem gátolhatja a fiókokat.</x:v>
+        <x:v>Fehér/kréta alacsony ágytest megtartva; oldalfiók helyett felnyíló tároló</x:v>
       </x:c>
       <x:c r="AB44" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -34099,11 +34429,11 @@
         <x:v>Matrac külön; fióknyitás, éjjeli ütközés, 202cm külső hossz ellenőrzése.</x:v>
       </x:c>
       <x:c r="AG44" s="20" t="n">
-        <x:v>189900</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="AH44" s="21" t="n">
         <x:f>O44*AG44+SUM(R44:T44)</x:f>
-        <x:v>189900</x:v>
+        <x:v>250000</x:v>
       </x:c>
       <x:c r="AI44" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -34121,19 +34451,19 @@
         <x:v>PENDING</x:v>
       </x:c>
       <x:c r="AN44" s="1" t="str">
-        <x:v>KI-043</x:v>
+        <x:v>BED-01</x:v>
       </x:c>
       <x:c r="AO44" s="1" t="str">
-        <x:v>drawings/P-01_alaprajz.pdf</x:v>
+        <x:v>R06/drawings/R06_valtozott_szerkezetek.pdf</x:v>
       </x:c>
       <x:c r="AP44" s="1" t="str">
-        <x:v>KI_KI-043</x:v>
+        <x:v>R06_BED01_*</x:v>
       </x:c>
       <x:c r="AQ44" s="1" t="str">
-        <x:v>késztermék / szakági munka</x:v>
+        <x:v>Egyedi</x:v>
       </x:c>
       <x:c r="AR44" s="1" t="str">
-        <x:v>felmérés/gyártói rajz szükséges</x:v>
+        <x:v>Tervezési befoglaló; vasalat és gyártás nincs jóváhagyva</x:v>
       </x:c>
       <x:c r="AS44" s="1" t="str">
         <x:v>HUF</x:v>
@@ -34154,18 +34484,18 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="AY44" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="AZ44" s="1" t="n">
-        <x:v>1.12</x:v>
+        <x:v>1.45</x:v>
       </x:c>
       <x:c r="BA44" s="29" t="n">
         <x:f>ROUND(U44*AY44,0)</x:f>
-        <x:v>189900</x:v>
+        <x:v>212500</x:v>
       </x:c>
       <x:c r="BB44" s="29" t="n">
         <x:f>ROUND(U44*AZ44,0)</x:f>
-        <x:v>212688</x:v>
+        <x:v>362500</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="72" customHeight="1">
@@ -34194,16 +34524,16 @@
         <x:v>180×200 matrac</x:v>
       </x:c>
       <x:c r="I45" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>IKEA</x:v>
       </x:c>
       <x:c r="J45" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>004.507.57</x:v>
       </x:c>
       <x:c r="K45" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>https://www.ikea.com/hu/hu/p/vagstranda-zsakrugos-matrac-kemeny-vilagoskek-00450757/</x:v>
       </x:c>
       <x:c r="L45" s="19" t="str">
-        <x:v>UNKNOWN – felmérés/gyári adat kell</x:v>
+        <x:v>1800×2000×280 mm</x:v>
       </x:c>
       <x:c r="M45" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -34218,7 +34548,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q45" s="20" t="n">
-        <x:v>260000</x:v>
+        <x:v>229900</x:v>
       </x:c>
       <x:c r="R45" s="20" t="n">
         <x:v>0</x:v>
@@ -34231,16 +34561,16 @@
       </x:c>
       <x:c r="U45" s="21" t="n">
         <x:f>O45*Q45+SUM(R45:T45)</x:f>
-        <x:v>260000</x:v>
+        <x:v>229900</x:v>
       </x:c>
       <x:c r="V45" s="19" t="str">
-        <x:v>előzetes becslés</x:v>
+        <x:v>Ellenőrzött webshopár</x:v>
       </x:c>
       <x:c r="W45" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 04a</x:v>
+        <x:v>IKEA HU 2026-10-27; komfortpróba és szállítás visszaigazolása nincs</x:v>
       </x:c>
       <x:c r="X45" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="Y45" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -34267,11 +34597,11 @@
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
       </x:c>
       <x:c r="AG45" s="20" t="n">
-        <x:v>260000</x:v>
+        <x:v>229900</x:v>
       </x:c>
       <x:c r="AH45" s="21" t="n">
         <x:f>O45*AG45+SUM(R45:T45)</x:f>
-        <x:v>260000</x:v>
+        <x:v>229900</x:v>
       </x:c>
       <x:c r="AI45" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -34329,11 +34659,11 @@
       </x:c>
       <x:c r="BA45" s="29" t="n">
         <x:f>ROUND(U45*AY45,0)</x:f>
-        <x:v>221000</x:v>
+        <x:v>195415</x:v>
       </x:c>
       <x:c r="BB45" s="29" t="n">
         <x:f>ROUND(U45*AZ45,0)</x:f>
-        <x:v>338000</x:v>
+        <x:v>298870</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="72" customHeight="1">
@@ -35363,7 +35693,7 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H52" s="19" t="str">
-        <x:v>Grafikás frontok és pántok</x:v>
+        <x:v>Északi és déli teljes magasságú grafikás frontok és pántok</x:v>
       </x:c>
       <x:c r="I52" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -35390,7 +35720,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q52" s="20" t="n">
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="R52" s="20" t="n">
         <x:v>0</x:v>
@@ -35403,13 +35733,13 @@
       </x:c>
       <x:c r="U52" s="21" t="n">
         <x:f>O52*Q52+SUM(R52:T52)</x:f>
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="V52" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W52" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 04c</x:v>
+        <x:v>Korábbi370000+80000 előirányzat a déli négy hosszú front merevítésére/pántolására; gyártói árajánlat szükséges</x:v>
       </x:c>
       <x:c r="X52" s="19" t="str">
         <x:v>2026-10-26</x:v>
@@ -35421,7 +35751,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="AA52" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>Észak6 és dél4 folytonos magas front; délen hosszú fekete fogantyú; eredeti grafika helyett R06 próbaváltozat</x:v>
       </x:c>
       <x:c r="AB52" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -35439,11 +35769,11 @@
         <x:v>6×2837 mm magas keskeny északi front. 250000+120000 becslés. Merevítés és műhelyméret nyitott.</x:v>
       </x:c>
       <x:c r="AG52" s="20" t="n">
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="AH52" s="21" t="n">
         <x:f>O52*AG52+SUM(R52:T52)</x:f>
-        <x:v>370000</x:v>
+        <x:v>450000</x:v>
       </x:c>
       <x:c r="AI52" s="19" t="str">
         <x:v>R05 főváltozat tartalma; korábbi fiók-/aszimmetria-elhagyás nincs automatikusan kiválasztva.</x:v>
@@ -35464,7 +35794,7 @@
         <x:v>WN-01; WS-01</x:v>
       </x:c>
       <x:c r="AO52" s="1" t="str">
-        <x:v>CP3/drawings/WN-01_CP3.pdf; CP3/drawings/WS-01_CP3.pdf</x:v>
+        <x:v>R06/drawings/R06_valtozott_szerkezetek.pdf</x:v>
       </x:c>
       <x:c r="AP52" s="1" t="str">
         <x:v>CP3_WN-01; CP3_WS-01</x:v>
@@ -35501,11 +35831,11 @@
       </x:c>
       <x:c r="BA52" s="29" t="n">
         <x:f>ROUND(U52*AY52,0)</x:f>
-        <x:v>277500</x:v>
+        <x:v>337500</x:v>
       </x:c>
       <x:c r="BB52" s="29" t="n">
         <x:f>ROUND(U52*AZ52,0)</x:f>
-        <x:v>573500</x:v>
+        <x:v>697500</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="72" customHeight="1">
@@ -39636,7 +39966,7 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF77" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>R06: változatlan350×350×450 test; új helyX14025,Y5920mm. Fiók/ajtó mozgás részletesen ellenőrzendő.</x:v>
       </x:c>
       <x:c r="AG77" s="20" t="n">
         <x:v>35000</x:v>
@@ -42156,7 +42486,7 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF92" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>R06: északi zuhanytálca déli élén keleti1000mm fixüveg,780mm névleges belépő. Kiviteli helyszíni vízzárás/üvegméret szakági jóváhagyásra vár.</x:v>
       </x:c>
       <x:c r="AG92" s="20" t="n">
         <x:v>180000</x:v>
@@ -45165,7 +45495,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="AA110" s="19" t="str">
-        <x:v>A render papírszerű, lágy lanternahatása közeli, a valós anyag szintetikus rost. Ø75/76 forrásellentmondás.</x:v>
+        <x:v>A gyári Somar laposabb búra, mint a konyhai render felfújt gömbje; a render igazodjon a gyárihoz.</x:v>
       </x:c>
       <x:c r="AB110" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -45211,13 +45541,13 @@
         <x:v>drawings/P-01_alaprajz.pdf</x:v>
       </x:c>
       <x:c r="AP110" s="1" t="str">
-        <x:v>NINCS MODELL / nem térbeli költségsor; szakági kapcsolat igazolandó</x:v>
+        <x:v>R06_Somar_*</x:v>
       </x:c>
       <x:c r="AQ110" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
       </x:c>
       <x:c r="AR110" s="1" t="str">
-        <x:v>felmérés/gyártói rajz szükséges</x:v>
+        <x:v>Ø760×360mm búra, E27; fotó alapján rekonstruált bordás forma</x:v>
       </x:c>
       <x:c r="AS110" s="1" t="str">
         <x:v>HUF</x:v>
@@ -46451,19 +46781,19 @@
         <x:v>Villamos</x:v>
       </x:c>
       <x:c r="H118" s="19" t="str">
-        <x:v>2×FADO fehér opálgömb + 2×Hue E27</x:v>
+        <x:v>2×EGLO RONDO 85264 Ø200 opálgömb + 2×Hue E27</x:v>
       </x:c>
       <x:c r="I118" s="19" t="str">
-        <x:v>IKEA</x:v>
+        <x:v>EGLO</x:v>
       </x:c>
       <x:c r="J118" s="19" t="str">
-        <x:v>800.963.72 + Hue E27 variáns PENDING</x:v>
+        <x:v>85264</x:v>
       </x:c>
       <x:c r="K118" s="19" t="str">
-        <x:v>https://www.ikea.com/hu/hu/p/fado-asztali-lampa-feher-80096372/</x:v>
+        <x:v>https://www.egloshop.hu/85264-eglo-rondo-asztali-lampa</x:v>
       </x:c>
       <x:c r="L118" s="19" t="str">
-        <x:v>Ø250×240 mm; 2 darab</x:v>
+        <x:v>Ø200×200 mm; E27</x:v>
       </x:c>
       <x:c r="M118" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -46478,7 +46808,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q118" s="20" t="n">
-        <x:v>11980</x:v>
+        <x:v>21980</x:v>
       </x:c>
       <x:c r="R118" s="20" t="n">
         <x:v>0</x:v>
@@ -46491,16 +46821,16 @@
       </x:c>
       <x:c r="U118" s="21" t="n">
         <x:f>O118*Q118+SUM(R118:T118)</x:f>
-        <x:v>35980</x:v>
+        <x:v>45980</x:v>
       </x:c>
       <x:c r="V118" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W118" s="19" t="str">
-        <x:v>https://www.ikea.com/hu/hu/p/fado-asztali-lampa-feher-80096372/</x:v>
+        <x:v>2×10990 Ft ellenőrzött lámpaár; 24000 Ft Hue előirányzat változatlan</x:v>
       </x:c>
       <x:c r="X118" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="Y118" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -46509,7 +46839,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="AA118" s="19" t="str">
-        <x:v>2×5990 Ft igazolt test + 24000 Ft becsült Hue izzópár. A célképnél nagyobb gömb, nincs magas fém talp. Beférés próba kötelező.</x:v>
+        <x:v>Kisebb gömb közelebb áll a célképhez; fehér talp a sötét referencia helyett.</x:v>
       </x:c>
       <x:c r="AB118" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -46527,11 +46857,11 @@
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
       </x:c>
       <x:c r="AG118" s="20" t="n">
-        <x:v>11980</x:v>
+        <x:v>21980</x:v>
       </x:c>
       <x:c r="AH118" s="21" t="n">
         <x:f>O118*AG118+SUM(R118:T118)</x:f>
-        <x:v>35980</x:v>
+        <x:v>45980</x:v>
       </x:c>
       <x:c r="AI118" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -46589,11 +46919,11 @@
       </x:c>
       <x:c r="BA118" s="29" t="n">
         <x:f>ROUND(U118*AY118,0)</x:f>
-        <x:v>35980</x:v>
+        <x:v>45980</x:v>
       </x:c>
       <x:c r="BB118" s="29" t="n">
         <x:f>ROUND(U118*AZ118,0)</x:f>
-        <x:v>40298</x:v>
+        <x:v>51498</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="72" customHeight="1">
@@ -56094,6 +56424,456 @@
       <x:c r="BB175" s="29" t="n">
         <x:f>ROUND(U175*AZ175,0)</x:f>
         <x:v>120000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="12" t="str">
+        <x:v>A902</x:v>
+      </x:c>
+      <x:c r="B176" s="12" t="str">
+        <x:v>06.2</x:v>
+      </x:c>
+      <x:c r="C176" s="12" t="str">
+        <x:v>KI-R06-01</x:v>
+      </x:c>
+      <x:c r="D176" s="12" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="E176" s="12" t="str">
+        <x:v>R06 új célkép</x:v>
+      </x:c>
+      <x:c r="F176" s="12" t="str">
+        <x:v>Stílus</x:v>
+      </x:c>
+      <x:c r="G176" s="12" t="str">
+        <x:v>Asztalos / szakági</x:v>
+      </x:c>
+      <x:c r="H176" s="19" t="str">
+        <x:v>06.2 WC feletti lamellás tölgyhatású tároló, világított fülkével</x:v>
+      </x:c>
+      <x:c r="I176" s="19" t="str">
+        <x:v>Ajánlatkérés</x:v>
+      </x:c>
+      <x:c r="J176" s="19" t="str">
+        <x:v>B62-WC-R06</x:v>
+      </x:c>
+      <x:c r="K176" s="19"/>
+      <x:c r="L176" s="19" t="str">
+        <x:v>900×200×1400mm; z1300;600ajtó+300nyitottfülke. Korpusz45000+front/lamella65000+vasalat20000+LED/táp25000+szerelés65000.</x:v>
+      </x:c>
+      <x:c r="M176" s="19"/>
+      <x:c r="N176" s="19"/>
+      <x:c r="O176" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P176" s="19" t="str">
+        <x:v>csomag</x:v>
+      </x:c>
+      <x:c r="Q176" s="20" t="n">
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="R176" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S176" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T176" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U176" s="21" t="n">
+        <x:f>O176*Q176+SUM(R176:T176)</x:f>
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="V176" s="19" t="str">
+        <x:v>Becslés</x:v>
+      </x:c>
+      <x:c r="W176" s="19" t="str">
+        <x:v>900×200×1400mm; z1300;600ajtó+300nyitottfülke. Korpusz45000+front/lamella65000+vasalat20000+LED/táp25000+szerelés65000.</x:v>
+      </x:c>
+      <x:c r="X176" s="19" t="str">
+        <x:v>2026-10-27</x:v>
+      </x:c>
+      <x:c r="Y176" s="19" t="str">
+        <x:v>6–10 hét feltételes</x:v>
+      </x:c>
+      <x:c r="Z176" s="19"/>
+      <x:c r="AA176" s="19" t="str">
+        <x:v>T07 alapján, hiteles geometria miatti eltérés dokumentálva</x:v>
+      </x:c>
+      <x:c r="AB176" s="19" t="str">
+        <x:v>Tervjavaslat, nem gyártási jóváhagyás</x:v>
+      </x:c>
+      <x:c r="AC176" s="19" t="str">
+        <x:v>Nincs megrendelve</x:v>
+      </x:c>
+      <x:c r="AD176" s="19" t="str">
+        <x:v>Asztalos / szakági tervező</x:v>
+      </x:c>
+      <x:c r="AE176" s="19"/>
+      <x:c r="AF176" s="19" t="str">
+        <x:v>900×200×1400mm; z1300;600ajtó+300nyitottfülke. Korpusz45000+front/lamella65000+vasalat20000+LED/táp25000+szerelés65000.</x:v>
+      </x:c>
+      <x:c r="AG176" s="20" t="n">
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="AH176" s="21" t="n">
+        <x:f>O176*AG176+SUM(R176:T176)</x:f>
+        <x:v>220000</x:v>
+      </x:c>
+      <x:c r="AI176" s="19" t="str">
+        <x:v>Tartalom megőrizve</x:v>
+      </x:c>
+      <x:c r="AJ176" s="19"/>
+      <x:c r="AK176" s="19"/>
+      <x:c r="AL176" s="19"/>
+      <x:c r="AM176" s="19"/>
+      <x:c r="AN176" s="1" t="str">
+        <x:v>B62-WC</x:v>
+      </x:c>
+      <x:c r="AO176" s="1" t="str">
+        <x:v>R06/drawings/R06_valtozott_szerkezetek.pdf</x:v>
+      </x:c>
+      <x:c r="AP176" s="1" t="str">
+        <x:v>R06_B62-WC*</x:v>
+      </x:c>
+      <x:c r="AQ176" s="1" t="str">
+        <x:v>Egyedi / jelölt</x:v>
+      </x:c>
+      <x:c r="AR176" s="1" t="str">
+        <x:v>Tervi, felmérés szükséges</x:v>
+      </x:c>
+      <x:c r="AS176" s="1" t="str">
+        <x:v>HUF</x:v>
+      </x:c>
+      <x:c r="AT176" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU176" s="1" t="str">
+        <x:v>Nem ajánlat</x:v>
+      </x:c>
+      <x:c r="AV176" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW176" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AX176" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY176" s="1" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AZ176" s="1" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="BA176" s="29" t="n">
+        <x:f>ROUND(U176*AY176,0)</x:f>
+        <x:v>176000</x:v>
+      </x:c>
+      <x:c r="BB176" s="29" t="n">
+        <x:f>ROUND(U176*AZ176,0)</x:f>
+        <x:v>330000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="12" t="str">
+        <x:v>A902</x:v>
+      </x:c>
+      <x:c r="B177" s="12" t="str">
+        <x:v>06.2</x:v>
+      </x:c>
+      <x:c r="C177" s="12" t="str">
+        <x:v>KI-R06-02</x:v>
+      </x:c>
+      <x:c r="D177" s="12" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="E177" s="12" t="str">
+        <x:v>R06 új célkép</x:v>
+      </x:c>
+      <x:c r="F177" s="12" t="str">
+        <x:v>Stílus</x:v>
+      </x:c>
+      <x:c r="G177" s="12" t="str">
+        <x:v>Asztalos / szakági</x:v>
+      </x:c>
+      <x:c r="H177" s="19" t="str">
+        <x:v>06.2 ág motívumos vízálló művészeti felület</x:v>
+      </x:c>
+      <x:c r="I177" s="19" t="str">
+        <x:v>Ajánlatkérés</x:v>
+      </x:c>
+      <x:c r="J177" s="19" t="str">
+        <x:v>ART-B62-R06</x:v>
+      </x:c>
+      <x:c r="K177" s="19"/>
+      <x:c r="L177" s="19" t="str">
+        <x:v>900×2400mm tervi felület; 2.16m²+15%rendelési ráhagyás. Védett hátoldali nyomat, üveg/szakági rendszer50000+grafika/nyomat25000+rögzítés35000. Zuhanyzónában akasztó/pad nem kerülhet elé.</x:v>
+      </x:c>
+      <x:c r="M177" s="19"/>
+      <x:c r="N177" s="19"/>
+      <x:c r="O177" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P177" s="19" t="str">
+        <x:v>csomag</x:v>
+      </x:c>
+      <x:c r="Q177" s="20" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="R177" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S177" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T177" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U177" s="21" t="n">
+        <x:f>O177*Q177+SUM(R177:T177)</x:f>
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="V177" s="19" t="str">
+        <x:v>Becslés</x:v>
+      </x:c>
+      <x:c r="W177" s="19" t="str">
+        <x:v>900×2400mm tervi felület; 2.16m²+15%rendelési ráhagyás. Védett hátoldali nyomat, üveg/szakági rendszer50000+grafika/nyomat25000+rögzítés35000. Zuhanyzónában akasztó/pad nem kerülhet elé.</x:v>
+      </x:c>
+      <x:c r="X177" s="19" t="str">
+        <x:v>2026-10-27</x:v>
+      </x:c>
+      <x:c r="Y177" s="19" t="str">
+        <x:v>6–10 hét feltételes</x:v>
+      </x:c>
+      <x:c r="Z177" s="19"/>
+      <x:c r="AA177" s="19" t="str">
+        <x:v>T07 alapján, hiteles geometria miatti eltérés dokumentálva</x:v>
+      </x:c>
+      <x:c r="AB177" s="19" t="str">
+        <x:v>Tervjavaslat, nem gyártási jóváhagyás</x:v>
+      </x:c>
+      <x:c r="AC177" s="19" t="str">
+        <x:v>Nincs megrendelve</x:v>
+      </x:c>
+      <x:c r="AD177" s="19" t="str">
+        <x:v>Asztalos / szakági tervező</x:v>
+      </x:c>
+      <x:c r="AE177" s="19"/>
+      <x:c r="AF177" s="19" t="str">
+        <x:v>900×2400mm tervi felület; 2.16m²+15%rendelési ráhagyás. Védett hátoldali nyomat, üveg/szakági rendszer50000+grafika/nyomat25000+rögzítés35000. Zuhanyzónában akasztó/pad nem kerülhet elé.</x:v>
+      </x:c>
+      <x:c r="AG177" s="20" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="AH177" s="21" t="n">
+        <x:f>O177*AG177+SUM(R177:T177)</x:f>
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="AI177" s="19" t="str">
+        <x:v>Tartalom megőrizve</x:v>
+      </x:c>
+      <x:c r="AJ177" s="19"/>
+      <x:c r="AK177" s="19"/>
+      <x:c r="AL177" s="19"/>
+      <x:c r="AM177" s="19"/>
+      <x:c r="AN177" s="1" t="str">
+        <x:v>ART-B62</x:v>
+      </x:c>
+      <x:c r="AO177" s="1" t="str">
+        <x:v>R06/drawings/R06_valtozott_szerkezetek.pdf</x:v>
+      </x:c>
+      <x:c r="AP177" s="1" t="str">
+        <x:v>R06_ART-B62*</x:v>
+      </x:c>
+      <x:c r="AQ177" s="1" t="str">
+        <x:v>Egyedi / jelölt</x:v>
+      </x:c>
+      <x:c r="AR177" s="1" t="str">
+        <x:v>Tervi, felmérés szükséges</x:v>
+      </x:c>
+      <x:c r="AS177" s="1" t="str">
+        <x:v>HUF</x:v>
+      </x:c>
+      <x:c r="AT177" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU177" s="1" t="str">
+        <x:v>Nem ajánlat</x:v>
+      </x:c>
+      <x:c r="AV177" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW177" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AX177" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY177" s="1" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AZ177" s="1" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="BA177" s="29" t="n">
+        <x:f>ROUND(U177*AY177,0)</x:f>
+        <x:v>88000</x:v>
+      </x:c>
+      <x:c r="BB177" s="29" t="n">
+        <x:f>ROUND(U177*AZ177,0)</x:f>
+        <x:v>165000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="12" t="str">
+        <x:v>A902</x:v>
+      </x:c>
+      <x:c r="B178" s="12" t="str">
+        <x:v>06.2</x:v>
+      </x:c>
+      <x:c r="C178" s="12" t="str">
+        <x:v>KI-R06-03</x:v>
+      </x:c>
+      <x:c r="D178" s="12" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="E178" s="12" t="str">
+        <x:v>R06 új célkép</x:v>
+      </x:c>
+      <x:c r="F178" s="12" t="str">
+        <x:v>Stílus</x:v>
+      </x:c>
+      <x:c r="G178" s="12" t="str">
+        <x:v>Asztalos / szakági</x:v>
+      </x:c>
+      <x:c r="H178" s="19" t="str">
+        <x:v>06.2 fekete törölközőszárító és csatlakozás előirányzat</x:v>
+      </x:c>
+      <x:c r="I178" s="19" t="str">
+        <x:v>Ajánlatkérés</x:v>
+      </x:c>
+      <x:c r="J178" s="19" t="str">
+        <x:v>RAD-B62-R06</x:v>
+      </x:c>
+      <x:c r="K178" s="19"/>
+      <x:c r="L178" s="19" t="str">
+        <x:v>400×1200mm tervi befoglaló; késztermék70000+bekötés/rögzítés50000. Pontos modell, hőigény, zóna és kiállás nyitott; meglévő esetén csak igazolás után levonható.</x:v>
+      </x:c>
+      <x:c r="M178" s="19"/>
+      <x:c r="N178" s="19"/>
+      <x:c r="O178" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P178" s="19" t="str">
+        <x:v>csomag</x:v>
+      </x:c>
+      <x:c r="Q178" s="20" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="R178" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S178" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T178" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U178" s="21" t="n">
+        <x:f>O178*Q178+SUM(R178:T178)</x:f>
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="V178" s="19" t="str">
+        <x:v>Becslés</x:v>
+      </x:c>
+      <x:c r="W178" s="19" t="str">
+        <x:v>400×1200mm tervi befoglaló; késztermék70000+bekötés/rögzítés50000. Pontos modell, hőigény, zóna és kiállás nyitott; meglévő esetén csak igazolás után levonható.</x:v>
+      </x:c>
+      <x:c r="X178" s="19" t="str">
+        <x:v>2026-10-27</x:v>
+      </x:c>
+      <x:c r="Y178" s="19" t="str">
+        <x:v>6–10 hét feltételes</x:v>
+      </x:c>
+      <x:c r="Z178" s="19"/>
+      <x:c r="AA178" s="19" t="str">
+        <x:v>T07 alapján, hiteles geometria miatti eltérés dokumentálva</x:v>
+      </x:c>
+      <x:c r="AB178" s="19" t="str">
+        <x:v>Tervjavaslat, nem gyártási jóváhagyás</x:v>
+      </x:c>
+      <x:c r="AC178" s="19" t="str">
+        <x:v>Nincs megrendelve</x:v>
+      </x:c>
+      <x:c r="AD178" s="19" t="str">
+        <x:v>Asztalos / szakági tervező</x:v>
+      </x:c>
+      <x:c r="AE178" s="19"/>
+      <x:c r="AF178" s="19" t="str">
+        <x:v>400×1200mm tervi befoglaló; késztermék70000+bekötés/rögzítés50000. Pontos modell, hőigény, zóna és kiállás nyitott; meglévő esetén csak igazolás után levonható.</x:v>
+      </x:c>
+      <x:c r="AG178" s="20" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="AH178" s="21" t="n">
+        <x:f>O178*AG178+SUM(R178:T178)</x:f>
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="AI178" s="19" t="str">
+        <x:v>Tartalom megőrizve</x:v>
+      </x:c>
+      <x:c r="AJ178" s="19"/>
+      <x:c r="AK178" s="19"/>
+      <x:c r="AL178" s="19"/>
+      <x:c r="AM178" s="19"/>
+      <x:c r="AN178" s="1" t="str">
+        <x:v>RAD-B62</x:v>
+      </x:c>
+      <x:c r="AO178" s="1" t="str">
+        <x:v>R06/drawings/R06_valtozott_szerkezetek.pdf</x:v>
+      </x:c>
+      <x:c r="AP178" s="1" t="str">
+        <x:v>R06_RAD-B62*</x:v>
+      </x:c>
+      <x:c r="AQ178" s="1" t="str">
+        <x:v>Egyedi / jelölt</x:v>
+      </x:c>
+      <x:c r="AR178" s="1" t="str">
+        <x:v>Tervi, felmérés szükséges</x:v>
+      </x:c>
+      <x:c r="AS178" s="1" t="str">
+        <x:v>HUF</x:v>
+      </x:c>
+      <x:c r="AT178" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU178" s="1" t="str">
+        <x:v>Nem ajánlat</x:v>
+      </x:c>
+      <x:c r="AV178" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW178" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AX178" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY178" s="1" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AZ178" s="1" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="BA178" s="29" t="n">
+        <x:f>ROUND(U178*AY178,0)</x:f>
+        <x:v>96000</x:v>
+      </x:c>
+      <x:c r="BB178" s="29" t="n">
+        <x:f>ROUND(U178*AZ178,0)</x:f>
+        <x:v>180000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -56107,7 +56887,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5789f99e06bb4575"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1a3955fcbed43fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -56159,11 +56939,11 @@
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A2)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A2)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="E2" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A2)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A2)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
@@ -56185,11 +56965,11 @@
         <x:v>1100000</x:v>
       </x:c>
       <x:c r="D3" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A3)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A3)</x:f>
         <x:v>1285000</x:v>
       </x:c>
       <x:c r="E3" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A3)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A3)</x:f>
         <x:v>1285000</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
@@ -56211,11 +56991,11 @@
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A4)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A4)</x:f>
         <x:v>252990</x:v>
       </x:c>
       <x:c r="E4" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A4)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A4)</x:f>
         <x:v>252990</x:v>
       </x:c>
       <x:c r="F4" s="18" t="n">
@@ -56237,11 +57017,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D5" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A5)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A5)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="E5" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A5)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A5)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="F5" s="18" t="n">
@@ -56263,11 +57043,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D6" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A6)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A6)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="E6" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A6)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A6)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="F6" s="18" t="n">
@@ -56289,11 +57069,11 @@
         <x:v>500000</x:v>
       </x:c>
       <x:c r="D7" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A7)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A7)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="E7" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A7)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A7)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="F7" s="18" t="n">
@@ -56315,11 +57095,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D8" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A8)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A8)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="E8" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A8)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A8)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="F8" s="18" t="n">
@@ -56341,11 +57121,11 @@
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="D9" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A9)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A9)</x:f>
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A9)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A9)</x:f>
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="F9" s="18" t="n">
@@ -56367,11 +57147,11 @@
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D10" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A10)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A10)</x:f>
         <x:v>300000</x:v>
       </x:c>
       <x:c r="E10" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A10)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A10)</x:f>
         <x:v>300000</x:v>
       </x:c>
       <x:c r="F10" s="18" t="n">
@@ -56393,11 +57173,11 @@
         <x:v>600000</x:v>
       </x:c>
       <x:c r="D11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A11)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A11)</x:f>
         <x:v>600000</x:v>
       </x:c>
       <x:c r="E11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A11)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A11)</x:f>
         <x:v>600000</x:v>
       </x:c>
       <x:c r="F11" s="18" t="n">
@@ -56419,11 +57199,11 @@
         <x:v>550000</x:v>
       </x:c>
       <x:c r="D12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A12)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A12)</x:f>
         <x:v>550000</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A12)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A12)</x:f>
         <x:v>550000</x:v>
       </x:c>
       <x:c r="F12" s="18" t="n">
@@ -56445,11 +57225,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D13" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A13)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A13)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="E13" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A13)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A13)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="F13" s="18" t="n">
@@ -56471,11 +57251,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A14)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A14)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="E14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A14)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A14)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="F14" s="18" t="n">
@@ -56497,11 +57277,11 @@
         <x:v>1189000</x:v>
       </x:c>
       <x:c r="D15" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A15)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A15)</x:f>
         <x:v>1450000</x:v>
       </x:c>
       <x:c r="E15" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A15)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A15)</x:f>
         <x:v>1450000</x:v>
       </x:c>
       <x:c r="F15" s="18" t="n">
@@ -56523,11 +57303,11 @@
         <x:v>861000</x:v>
       </x:c>
       <x:c r="D16" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A16)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A16)</x:f>
         <x:v>1450000</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A16)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A16)</x:f>
         <x:v>1350000</x:v>
       </x:c>
       <x:c r="F16" s="18" t="n">
@@ -56549,11 +57329,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D17" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A17)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A17)</x:f>
         <x:v>800000</x:v>
       </x:c>
       <x:c r="E17" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A17)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A17)</x:f>
         <x:v>800000</x:v>
       </x:c>
       <x:c r="F17" s="18" t="n">
@@ -56575,11 +57355,11 @@
         <x:v>220000</x:v>
       </x:c>
       <x:c r="D18" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A18)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A18)</x:f>
         <x:v>160000</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A18)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A18)</x:f>
         <x:v>160000</x:v>
       </x:c>
       <x:c r="F18" s="18" t="n">
@@ -56601,11 +57381,11 @@
         <x:v>760000</x:v>
       </x:c>
       <x:c r="D19" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A19)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A19)</x:f>
         <x:v>711070</x:v>
       </x:c>
       <x:c r="E19" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A19)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A19)</x:f>
         <x:v>711070</x:v>
       </x:c>
       <x:c r="F19" s="18" t="n">
@@ -56627,11 +57407,11 @@
         <x:v>200000</x:v>
       </x:c>
       <x:c r="D20" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A20)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A20)</x:f>
         <x:v>200000</x:v>
       </x:c>
       <x:c r="E20" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A20)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A20)</x:f>
         <x:v>200000</x:v>
       </x:c>
       <x:c r="F20" s="18" t="n">
@@ -56653,11 +57433,11 @@
         <x:v>260000</x:v>
       </x:c>
       <x:c r="D21" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A21)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A21)</x:f>
         <x:v>280000</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A21)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A21)</x:f>
         <x:v>280000</x:v>
       </x:c>
       <x:c r="F21" s="18" t="n">
@@ -56679,16 +57459,16 @@
         <x:v>550000</x:v>
       </x:c>
       <x:c r="D22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A22)</x:f>
-        <x:v>469900</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A22)</x:f>
+        <x:v>499900</x:v>
       </x:c>
       <x:c r="E22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A22)</x:f>
-        <x:v>469900</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A22)</x:f>
+        <x:v>499900</x:v>
       </x:c>
       <x:c r="F22" s="18" t="n">
         <x:f>E22-C22</x:f>
-        <x:v>-80100</x:v>
+        <x:v>-50100</x:v>
       </x:c>
       <x:c r="G22" s="19" t="str">
         <x:v>180×200 ágykeret és tartóalap; 180×200 matrac; Matracvédő</x:v>
@@ -56705,11 +57485,11 @@
         <x:v>353000</x:v>
       </x:c>
       <x:c r="D23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A23)</x:f>
         <x:v>355000</x:v>
       </x:c>
       <x:c r="E23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A23)</x:f>
         <x:v>355000</x:v>
       </x:c>
       <x:c r="F23" s="18" t="n">
@@ -56731,16 +57511,16 @@
         <x:v>820000</x:v>
       </x:c>
       <x:c r="D24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A24)</x:f>
-        <x:v>1916000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A24)</x:f>
+        <x:v>1996000</x:v>
       </x:c>
       <x:c r="E24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A24)</x:f>
-        <x:v>1916000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A24)</x:f>
+        <x:v>1996000</x:v>
       </x:c>
       <x:c r="F24" s="18" t="n">
         <x:f>E24-C24</x:f>
-        <x:v>1096000</x:v>
+        <x:v>1176000</x:v>
       </x:c>
       <x:c r="G24" s="19" t="str">
         <x:v>Északi gardrób szabványkorpuszok; Déli gardrób szabványkorpuszok; Északi és déli gardróbbelsők; Grafikás frontok és pántok; Felső kitöltések, takarók, rögzítés és szerelés</x:v>
@@ -56757,11 +57537,11 @@
         <x:v>380000</x:v>
       </x:c>
       <x:c r="D25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A25)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="E25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A25)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="F25" s="18" t="n">
@@ -56783,11 +57563,11 @@
         <x:v>820000</x:v>
       </x:c>
       <x:c r="D26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A26)</x:f>
         <x:v>1085000</x:v>
       </x:c>
       <x:c r="E26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A26)</x:f>
         <x:v>1085000</x:v>
       </x:c>
       <x:c r="F26" s="18" t="n">
@@ -56809,16 +57589,16 @@
         <x:v>1400000</x:v>
       </x:c>
       <x:c r="D27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A27)</x:f>
-        <x:v>2050360</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A27)</x:f>
+        <x:v>2060360</x:v>
       </x:c>
       <x:c r="E27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A27)</x:f>
-        <x:v>2050360</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A27)</x:f>
+        <x:v>2060360</x:v>
       </x:c>
       <x:c r="F27" s="18" t="n">
         <x:f>E27-C27</x:f>
-        <x:v>650360</x:v>
+        <x:v>660360</x:v>
       </x:c>
       <x:c r="G27" s="19" t="str">
         <x:v>Hue Bridge és hálózati csatlakozás; Hue vezérlők és kapcsolómodulok; Villamos kábel, csatlakozó, doboz és kábelrejtés; Villanyszerelés, mérések, címkézés; Hue programozás, jelenetek, próbaüzem; Somar függeszték és Hue E27; Négy Hue-kompatibilis általános lámpatest/izzó; ML03 általános fény és FL01 falikar, Hue fényforrások; Pultvilágítás szalag, táp, vezérlő, profil és fedél; ML05 Hue mennyezeti lámpa; W01 felső, függőleges és alsó vonalfény komplett; W02/W07 grafikai falmosás komplett; ML06 mennyezeti Hue lámpa; Két éjjeli gömblámpa Hue fényforrással; Fejvég rejtett fénye szalag/táp/profil; Gardróbbelsők funkcionális fénye; Két fürdő mennyezeti és mosdó feletti gyári Hue lámpái; 06.2 két külön rejtett fény és védett szerelvényrendszer; Fürdő tápegységek száraz oldali szervizelhelyezése</x:v>
@@ -56835,11 +57615,11 @@
         <x:v>336000</x:v>
       </x:c>
       <x:c r="D28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A28)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="E28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A28)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="F28" s="18" t="n">
@@ -56861,11 +57641,11 @@
         <x:v>262000</x:v>
       </x:c>
       <x:c r="D29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A29)</x:f>
         <x:v>551000</x:v>
       </x:c>
       <x:c r="E29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A29)</x:f>
         <x:v>503000</x:v>
       </x:c>
       <x:c r="F29" s="18" t="n">
@@ -56887,11 +57667,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$175,'Elemregiszter'!$E$2:$E$175,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A30)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="E30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$175,'Elemregiszter'!$E$2:$E$175,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A30)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="F30" s="18" t="n">
@@ -56916,15 +57696,15 @@
       </x:c>
       <x:c r="D31" s="18" t="n">
         <x:f>SUM(D2:D30)</x:f>
-        <x:v>22383680</x:v>
+        <x:v>22503680</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
         <x:f>SUM(E2:E30)</x:f>
-        <x:v>22235680</x:v>
+        <x:v>22355680</x:v>
       </x:c>
       <x:c r="F31" s="18" t="n">
         <x:f>SUM(F2:F30)</x:f>
-        <x:v>4624680</x:v>
+        <x:v>4744680</x:v>
       </x:c>
       <x:c r="G31" s="19"/>
     </x:row>

</xml_diff>

<commit_message>
R10: rebuild 3600mm media wall, high curtains, costed conditional living pilot
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
@@ -2,30 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R36f923b2bd5c428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="R5a663db2597c42b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R6a5dbed989eb4e2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R00bc4a9d73304419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="Re2eddac4a63c4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="Rad3f698ce8b344e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="R247f37bcf5b84807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="R788bc37c0d80435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="R918c68f7a6924c54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="R33b845d9132045c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="R66fe7959d04545b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="Rc87a2cb0bbaa418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="Ra2d833928f994d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="R916d3c7ce21648d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="R90cba8e611bb4c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R2c972e89bad4460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="Recea1fd0f1f8420e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="R62314806f80b4a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="Rd089dc3f38fd44f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="R9ce53e5c38804796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R7744d4f00a18492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R11c0036e45f64e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="Rcd609916148c4f66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 változások" sheetId="24" r:id="Refa2a637b72244b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R824f5e37e7314c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="Re9de161a947c4ab7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R9dceecd1562548d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R16cf21137f82446c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="R04d67890da524bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="Rbc81d6d2a8a34243"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="R6e44304fd72a4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="Rf718dd1e79b64ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="R048b2710971d4a6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="R92812f3040a14b8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="R89f0fb5c34cc4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="R88e5401dc66249c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="R30a183406d444737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="Rf5ba364675f3465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="R5f757a4fff364951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R3d74062258c94d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="R75627b8a59e44fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="Rebd0add04ec04da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="R121bb85634de46fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="R977ff9c348a74821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R37d48707329c4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R4a47cf488fc248e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="Re05e8dfc69914f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 változások" sheetId="24" r:id="R51c0e764b322439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R10 változások" sheetId="25" r:id="R44cb221dc96e4e14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -101,7 +102,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -111,6 +112,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF303E3C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF303C3B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -191,7 +197,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="64">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -362,6 +368,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2874,11 +2886,11 @@
       </x:c>
       <x:c r="D31" s="19" t="n">
         <x:f>'Elemregiszter'!U31</x:f>
-        <x:v>690000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="E31" s="19" t="n">
         <x:f>D31-C31</x:f>
-        <x:v>380000</x:v>
+        <x:v>455500</x:v>
       </x:c>
       <x:c r="F31" s="19" t="str">
         <x:v>W01 V3.3 panelmező, grafikus torony: nagyobb folytonos grafika; 3600×2880 tervezési befoglaló</x:v>
@@ -2896,11 +2908,11 @@
       </x:c>
       <x:c r="D32" s="19" t="n">
         <x:f>'Elemregiszter'!U32</x:f>
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="E32" s="19" t="n">
         <x:f>D32-C32</x:f>
-        <x:v>110000</x:v>
+        <x:v>140000</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str">
         <x:v>W01 V3.3 folytonos alsó tároló: 3300×400×400, 5 front</x:v>
@@ -2918,11 +2930,11 @@
       </x:c>
       <x:c r="D33" s="19" t="n">
         <x:f>'Elemregiszter'!U33</x:f>
-        <x:v>120000</x:v>
+        <x:v>135000</x:v>
       </x:c>
       <x:c r="E33" s="19" t="n">
         <x:f>D33-C33</x:f>
-        <x:v>0</x:v>
+        <x:v>15000</x:v>
       </x:c>
       <x:c r="F33" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -3116,11 +3128,11 @@
       </x:c>
       <x:c r="D42" s="19" t="n">
         <x:f>'Elemregiszter'!U42</x:f>
-        <x:v>65000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="E42" s="19" t="n">
         <x:f>D42-C42</x:f>
-        <x:v>0</x:v>
+        <x:v>15000</x:v>
       </x:c>
       <x:c r="F42" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -3138,11 +3150,11 @@
       </x:c>
       <x:c r="D43" s="19" t="n">
         <x:f>'Elemregiszter'!U43</x:f>
-        <x:v>55000</x:v>
+        <x:v>65000</x:v>
       </x:c>
       <x:c r="E43" s="19" t="n">
         <x:f>D43-C43</x:f>
-        <x:v>0</x:v>
+        <x:v>10000</x:v>
       </x:c>
       <x:c r="F43" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -19691,11 +19703,11 @@
         <x:v>Fő előrejelzés</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:f>SUM('Elemregiszter'!U2:U178)</x:f>
-        <x:v>24482890</x:v>
+        <x:f>SUM('Elemregiszter'!U2:U179)</x:f>
+        <x:v>24673390</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>R06: hét új célkép; pontos termékformák, grafikapróbák, magas gardróbfrontok és T07 kiegészítések. Nem rendelési engedély.</x:v>
+        <x:v>R10:3600mm médiafal,120mm sáv, magas függöny, külön textilek. Becslések, nem jóváhagyott többletkeret.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -19703,8 +19715,8 @@
         <x:v>Gazdaságos javaslat</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:f>SUM('Elemregiszter'!AH2:AH178)</x:f>
-        <x:v>24229890</x:v>
+        <x:f>SUM('Elemregiszter'!AH2:AH179)</x:f>
+        <x:v>24520390</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
         <x:v>Összehasonlítható takarékos változat:253000Ft dokumentált megtakarítás;18M továbbra sem igazolt.</x:v>
@@ -19716,7 +19728,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>B7-B5</x:f>
-        <x:v>6482890</x:v>
+        <x:v>6673390</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19728,7 +19740,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>B8-B5</x:f>
-        <x:v>6229890</x:v>
+        <x:v>6520390</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19739,7 +19751,7 @@
         <x:v>Ellenőrzött webshopár rész</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!V2:V178,"ellenőrzött webshopár")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!U2:U179,'Elemregiszter'!V2:V179,"ellenőrzött webshopár")</x:f>
         <x:v>2142440</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
@@ -19751,7 +19763,7 @@
         <x:v>Beszállítói ajánlat rész</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!V2:V178,"beszállítói ajánlat")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!U2:U179,'Elemregiszter'!V2:V179,"beszállítói ajánlat")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
@@ -19764,7 +19776,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>B7-B11-B12</x:f>
-        <x:v>22340450</x:v>
+        <x:v>22530950</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>Minden nem igazolt ár</x:v>
@@ -19775,7 +19787,7 @@
         <x:v>Megrendelt érték</x:v>
       </x:c>
       <x:c r="B14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!U2:U178,'Elemregiszter'!AC2:AC178,"megrendelt")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!U2:U179,'Elemregiszter'!AC2:AC179,"megrendelt")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
@@ -19787,11 +19799,11 @@
         <x:v>Tételszám</x:v>
       </x:c>
       <x:c r="B15" s="18" t="n">
-        <x:f>COUNTA('Elemregiszter'!C2:C178)</x:f>
-        <x:v>177</x:v>
+        <x:f>COUNTA('Elemregiszter'!C2:C179)</x:f>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>177 költségsor; a külön2M tartalékból0Ft felhasználva.</x:v>
+        <x:v>178 költségsor;2M tartalék érintetlen; R09 45000Ft textildelta már beépítve.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -19847,11 +19859,11 @@
         <x:v>teljes lakás</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A22)</x:f>
         <x:v>1953790</x:v>
       </x:c>
       <x:c r="C22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A22)</x:f>
         <x:v>1953790</x:v>
       </x:c>
     </x:row>
@@ -19860,11 +19872,11 @@
         <x:v>02</x:v>
       </x:c>
       <x:c r="B23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A23)</x:f>
         <x:v>3287990</x:v>
       </x:c>
       <x:c r="C23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A23)</x:f>
         <x:v>3287990</x:v>
       </x:c>
     </x:row>
@@ -19873,11 +19885,11 @@
         <x:v>03</x:v>
       </x:c>
       <x:c r="B24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A24)</x:f>
         <x:v>971070</x:v>
       </x:c>
       <x:c r="C24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A24)</x:f>
         <x:v>971070</x:v>
       </x:c>
     </x:row>
@@ -19886,12 +19898,12 @@
         <x:v>04</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A25)</x:f>
-        <x:v>3742190</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A25)</x:f>
+        <x:v>3932690</x:v>
       </x:c>
       <x:c r="C25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A25)</x:f>
-        <x:v>3594190</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A25)</x:f>
+        <x:v>3884690</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
@@ -19899,11 +19911,11 @@
         <x:v>05.1</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A26)</x:f>
         <x:v>3805500</x:v>
       </x:c>
       <x:c r="C26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A26)</x:f>
         <x:v>3805500</x:v>
       </x:c>
     </x:row>
@@ -19912,11 +19924,11 @@
         <x:v>05.2</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A27)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="C27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A27)</x:f>
         <x:v>1179980</x:v>
       </x:c>
     </x:row>
@@ -19925,11 +19937,11 @@
         <x:v>05.3</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A28)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="C28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A28)</x:f>
         <x:v>1157380</x:v>
       </x:c>
     </x:row>
@@ -19938,11 +19950,11 @@
         <x:v>01</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A29)</x:f>
         <x:v>440000</x:v>
       </x:c>
       <x:c r="C29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A29)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A29)</x:f>
         <x:v>440000</x:v>
       </x:c>
     </x:row>
@@ -19951,11 +19963,11 @@
         <x:v>07</x:v>
       </x:c>
       <x:c r="B30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A30)</x:f>
         <x:v>40000</x:v>
       </x:c>
       <x:c r="C30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A30)</x:f>
         <x:v>40000</x:v>
       </x:c>
     </x:row>
@@ -19964,11 +19976,11 @@
         <x:v>06.1 / elhelyezés PENDING</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A31)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A31)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="C31" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A31)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A31)</x:f>
         <x:v>485000</x:v>
       </x:c>
     </x:row>
@@ -19977,11 +19989,11 @@
         <x:v>06.2</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A32)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A32)</x:f>
         <x:v>1385000</x:v>
       </x:c>
       <x:c r="C32" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A32)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A32)</x:f>
         <x:v>1280000</x:v>
       </x:c>
     </x:row>
@@ -19990,11 +20002,11 @@
         <x:v>06.1</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A33)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A33)</x:f>
         <x:v>255000</x:v>
       </x:c>
       <x:c r="C33" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A33)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A33)</x:f>
         <x:v>255000</x:v>
       </x:c>
     </x:row>
@@ -20003,11 +20015,11 @@
         <x:v>08</x:v>
       </x:c>
       <x:c r="B34" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A34)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A34)</x:f>
         <x:v>75000</x:v>
       </x:c>
       <x:c r="C34" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A34)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A34)</x:f>
         <x:v>75000</x:v>
       </x:c>
     </x:row>
@@ -20016,11 +20028,11 @@
         <x:v>06.1 / 06.2 / 08</x:v>
       </x:c>
       <x:c r="B35" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A35)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A35)</x:f>
         <x:v>35000</x:v>
       </x:c>
       <x:c r="C35" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A35)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A35)</x:f>
         <x:v>35000</x:v>
       </x:c>
     </x:row>
@@ -20029,11 +20041,11 @@
         <x:v>01 / 07 / 08</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A36)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A36)</x:f>
         <x:v>130000</x:v>
       </x:c>
       <x:c r="C36" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A36)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A36)</x:f>
         <x:v>130000</x:v>
       </x:c>
     </x:row>
@@ -20042,11 +20054,11 @@
         <x:v>06.1 / 06.2</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A37)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A37)</x:f>
         <x:v>340000</x:v>
       </x:c>
       <x:c r="C37" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A37)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A37)</x:f>
         <x:v>340000</x:v>
       </x:c>
     </x:row>
@@ -20055,11 +20067,11 @@
         <x:v>04 / 07</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A38)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A38)</x:f>
         <x:v>315000</x:v>
       </x:c>
       <x:c r="C38" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A38)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A38)</x:f>
         <x:v>315000</x:v>
       </x:c>
     </x:row>
@@ -20068,11 +20080,11 @@
         <x:v>09 terasz Ny</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A39)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A39)</x:f>
         <x:v>2000000</x:v>
       </x:c>
       <x:c r="C39" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A39)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A39)</x:f>
         <x:v>2000000</x:v>
       </x:c>
     </x:row>
@@ -20081,11 +20093,11 @@
         <x:v>10 terasz K</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A40)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A40)</x:f>
         <x:v>1150000</x:v>
       </x:c>
       <x:c r="C40" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A40)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A40)</x:f>
         <x:v>1150000</x:v>
       </x:c>
     </x:row>
@@ -20094,11 +20106,11 @@
         <x:v>09 / 10 / 11 / 12 / 13 kültér</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A41)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A41)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="C41" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A41)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A41)</x:f>
         <x:v>590000</x:v>
       </x:c>
     </x:row>
@@ -20107,11 +20119,11 @@
         <x:v>01 / 04</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A42)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A42)</x:f>
         <x:v>360000</x:v>
       </x:c>
       <x:c r="C42" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$B$2:$B$178,A42)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A42)</x:f>
         <x:v>360000</x:v>
       </x:c>
     </x:row>
@@ -20141,11 +20153,11 @@
         <x:v>Tervezés</x:v>
       </x:c>
       <x:c r="B46" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A46)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A46)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="C46" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A46)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A46)</x:f>
         <x:v>420000</x:v>
       </x:c>
     </x:row>
@@ -20154,12 +20166,12 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="B47" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A47)</x:f>
-        <x:v>6216000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A47)</x:f>
+        <x:v>6336500</x:v>
       </x:c>
       <x:c r="C47" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A47)</x:f>
-        <x:v>6116000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A47)</x:f>
+        <x:v>6336500</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="30" customHeight="1">
@@ -20167,11 +20179,11 @@
         <x:v>Gépek</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A48)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A48)</x:f>
         <x:v>1770000</x:v>
       </x:c>
       <x:c r="C48" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A48)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A48)</x:f>
         <x:v>1770000</x:v>
       </x:c>
     </x:row>
@@ -20180,11 +20192,11 @@
         <x:v>Vízszerelés</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A49)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A49)</x:f>
         <x:v>412990</x:v>
       </x:c>
       <x:c r="C49" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A49)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A49)</x:f>
         <x:v>412990</x:v>
       </x:c>
     </x:row>
@@ -20193,11 +20205,11 @@
         <x:v>Bútor</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A50)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A50)</x:f>
         <x:v>4928330</x:v>
       </x:c>
       <x:c r="C50" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A50)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A50)</x:f>
         <x:v>4928330</x:v>
       </x:c>
     </x:row>
@@ -20206,11 +20218,11 @@
         <x:v>Elektronika</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A51)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A51)</x:f>
         <x:v>680000</x:v>
       </x:c>
       <x:c r="C51" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A51)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A51)</x:f>
         <x:v>680000</x:v>
       </x:c>
     </x:row>
@@ -20219,12 +20231,12 @@
         <x:v>Textil</x:v>
       </x:c>
       <x:c r="B52" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A52)</x:f>
-        <x:v>1330000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A52)</x:f>
+        <x:v>1400000</x:v>
       </x:c>
       <x:c r="C52" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A52)</x:f>
-        <x:v>1330000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A52)</x:f>
+        <x:v>1400000</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="30" customHeight="1">
@@ -20232,11 +20244,11 @@
         <x:v>Művészet</x:v>
       </x:c>
       <x:c r="B53" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A53)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A53)</x:f>
         <x:v>611000</x:v>
       </x:c>
       <x:c r="C53" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A53)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A53)</x:f>
         <x:v>563000</x:v>
       </x:c>
     </x:row>
@@ -20245,11 +20257,11 @@
         <x:v>Villamos</x:v>
       </x:c>
       <x:c r="B54" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A54)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A54)</x:f>
         <x:v>2200360</x:v>
       </x:c>
       <x:c r="C54" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A54)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A54)</x:f>
         <x:v>2200360</x:v>
       </x:c>
     </x:row>
@@ -20258,11 +20270,11 @@
         <x:v>Üveges</x:v>
       </x:c>
       <x:c r="B55" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A55)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A55)</x:f>
         <x:v>180000</x:v>
       </x:c>
       <x:c r="C55" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A55)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A55)</x:f>
         <x:v>180000</x:v>
       </x:c>
     </x:row>
@@ -20271,11 +20283,11 @@
         <x:v>Kiegészítők</x:v>
       </x:c>
       <x:c r="B56" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A56)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A56)</x:f>
         <x:v>250000</x:v>
       </x:c>
       <x:c r="C56" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A56)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A56)</x:f>
         <x:v>250000</x:v>
       </x:c>
     </x:row>
@@ -20284,11 +20296,11 @@
         <x:v>Falfelület</x:v>
       </x:c>
       <x:c r="B57" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A57)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A57)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="C57" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A57)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A57)</x:f>
         <x:v>405000</x:v>
       </x:c>
     </x:row>
@@ -20297,11 +20309,11 @@
         <x:v>Kert és terasz</x:v>
       </x:c>
       <x:c r="B58" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A58)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A58)</x:f>
         <x:v>2590000</x:v>
       </x:c>
       <x:c r="C58" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A58)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A58)</x:f>
         <x:v>2590000</x:v>
       </x:c>
     </x:row>
@@ -20310,11 +20322,11 @@
         <x:v>Logisztika</x:v>
       </x:c>
       <x:c r="B59" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$G$2:$G$178,A59)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A59)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="C59" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$G$2:$G$178,A59)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A59)</x:f>
         <x:v>510000</x:v>
       </x:c>
     </x:row>
@@ -20344,11 +20356,11 @@
         <x:v>FIX</x:v>
       </x:c>
       <x:c r="B63" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$F$2:$F$178,A63)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$F$2:$F$179,A63)</x:f>
         <x:v>9510350</x:v>
       </x:c>
       <x:c r="C63" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$F$2:$F$178,A63)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$F$2:$F$179,A63)</x:f>
         <x:v>9510350</x:v>
       </x:c>
     </x:row>
@@ -20357,12 +20369,12 @@
         <x:v>STÍLUS</x:v>
       </x:c>
       <x:c r="B64" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$F$2:$F$178,A64)</x:f>
-        <x:v>12993330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$F$2:$F$179,A64)</x:f>
+        <x:v>13183830</x:v>
       </x:c>
       <x:c r="C64" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$F$2:$F$178,A64)</x:f>
-        <x:v>12845330</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$F$2:$F$179,A64)</x:f>
+        <x:v>13135830</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="30" customHeight="1">
@@ -20391,12 +20403,12 @@
         <x:v>nem megrendelt</x:v>
       </x:c>
       <x:c r="B68" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$AC$2:$AC$178,A68)</x:f>
-        <x:v>22503680</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$AC$2:$AC$179,A68)</x:f>
+        <x:v>22694180</x:v>
       </x:c>
       <x:c r="C68" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$AC$2:$AC$178,A68)</x:f>
-        <x:v>22355680</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$AC$2:$AC$179,A68)</x:f>
+        <x:v>22646180</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -20427,8 +20439,8 @@
         <x:v>Alsó sáv</x:v>
       </x:c>
       <x:c r="B74" s="30" t="n">
-        <x:f>SUM('Elemregiszter'!BA2:BA178)</x:f>
-        <x:v>20841595</x:v>
+        <x:f>SUM('Elemregiszter'!BA2:BA179)</x:f>
+        <x:v>20990870</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>Sorok alsó feltételezéseinek összege</x:v>
@@ -20439,8 +20451,8 @@
         <x:v>Felső sáv</x:v>
       </x:c>
       <x:c r="B75" s="30" t="n">
-        <x:f>SUM('Elemregiszter'!BB2:BB178)</x:f>
-        <x:v>32952998</x:v>
+        <x:f>SUM('Elemregiszter'!BB2:BB179)</x:f>
+        <x:v>33210947</x:v>
       </x:c>
       <x:c r="C75" t="str">
         <x:v>Sorok felső feltételezéseinek összege</x:v>
@@ -20463,7 +20475,7 @@
       </x:c>
       <x:c r="B77" s="30" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>253000</x:v>
+        <x:v>153000</x:v>
       </x:c>
       <x:c r="C77" t="str">
         <x:v>Bruttó projektkülönbség, változatlan közös logisztikával</x:v>
@@ -20485,7 +20497,7 @@
         <x:v>AT8-01</x:v>
       </x:c>
       <x:c r="B80" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A80)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A80)</x:f>
         <x:v>380990</x:v>
       </x:c>
       <x:c r="C80" t="str">
@@ -20497,7 +20509,7 @@
         <x:v>T-0-26</x:v>
       </x:c>
       <x:c r="B81" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A81)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A81)</x:f>
         <x:v>165000</x:v>
       </x:c>
       <x:c r="C81" t="str">
@@ -20509,7 +20521,7 @@
         <x:v>AT8-01 / T-0-26</x:v>
       </x:c>
       <x:c r="B82" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$B$2:$B$178,A82)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A82)</x:f>
         <x:v>174000</x:v>
       </x:c>
       <x:c r="C82" t="str">
@@ -20521,7 +20533,7 @@
         <x:v>Fagyasztó és kapcsolódó munka</x:v>
       </x:c>
       <x:c r="B83" s="30" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$C$2:$C$178,"KI-CP3-F01")+SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$C$2:$C$178,"KI-CP3-F02")</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$C$2:$C$179,"KI-CP3-F01")+SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$C$2:$C$179,"KI-CP3-F02")</x:f>
         <x:v>334990</x:v>
       </x:c>
       <x:c r="C83" t="str">
@@ -20534,7 +20546,7 @@
       </x:c>
       <x:c r="B84" s="30" t="n">
         <x:f>B7-B83</x:f>
-        <x:v>24147900</x:v>
+        <x:v>24338400</x:v>
       </x:c>
       <x:c r="C84" t="str">
         <x:v>Nem automatikusan kiválasztott megtakarítás</x:v>
@@ -23988,19 +24000,19 @@
       </x:c>
       <x:c r="C2" s="55" t="n">
         <x:f>'Elemregiszter'!U31</x:f>
-        <x:v>690000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="D2" s="55" t="n">
         <x:f>C2-B2</x:f>
-        <x:v>240000</x:v>
+        <x:v>315500</x:v>
       </x:c>
       <x:c r="E2" s="55" t="n">
         <x:f>'Elemregiszter'!AH31</x:f>
-        <x:v>590000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="F2" s="55" t="n">
         <x:f>C2-E2</x:f>
-        <x:v>100000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="19" t="str">
         <x:v>R04 médiafal +240000: 160000 felületi többlet és80000 grafika/minta; különbözeti becslés, nem új teljes csomag. Gazdaságos összehasonlítás külön.</x:v>
@@ -24015,15 +24027,15 @@
       </x:c>
       <x:c r="C3" s="55" t="n">
         <x:f>'Elemregiszter'!U32</x:f>
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="D3" s="55" t="n">
         <x:f>C3-B3</x:f>
-        <x:v>60000</x:v>
+        <x:v>90000</x:v>
       </x:c>
       <x:c r="E3" s="55" t="n">
         <x:f>'Elemregiszter'!AH32</x:f>
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="F3" s="55" t="n">
         <x:f>C3-E3</x:f>
@@ -27043,6 +27055,153 @@
       </x:c>
       <x:c r="E16" s="1" t="str">
         <x:v>400×1200mm tervi befoglaló; késztermék70000+bekötés/rögzítés50000. Pontos modell, hőigény, zóna és kiállás nyitott; meglévő esetén csak igazolás után levonható.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="95" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="65" customHeight="1">
+      <x:c r="A1" s="65" t="str">
+        <x:v>Elem</x:v>
+      </x:c>
+      <x:c r="B1" s="65" t="str">
+        <x:v>Előző Ft</x:v>
+      </x:c>
+      <x:c r="C1" s="65" t="str">
+        <x:v>R10 Ft</x:v>
+      </x:c>
+      <x:c r="D1" s="65" t="str">
+        <x:v>Változás Ft</x:v>
+      </x:c>
+      <x:c r="E1" s="65" t="str">
+        <x:v>Indok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="65" customHeight="1">
+      <x:c r="A2" s="1" t="str">
+        <x:v>KI-030</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="n">
+        <x:v>690000</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="n">
+        <x:f>'Elemregiszter'!U31</x:f>
+        <x:v>765500</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="n">
+        <x:f>C2-B2</x:f>
+        <x:v>75500</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>+75500Ft becslés:0,4194m² többletfelület kb10500Ft; köztes sáv25000; szélek/alkatrész10000; új hordozó/nyomatpróba30000. Nem ajánlat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="65" customHeight="1">
+      <x:c r="A3" s="1" t="str">
+        <x:v>KI-031</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="n">
+        <x:v>320000</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="n">
+        <x:f>'Elemregiszter'!U32</x:f>
+        <x:v>350000</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="n">
+        <x:f>C3-B3</x:f>
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>+30000Ft:300mm többlet korpusz/top/front, régi320000×3600/3300≈349091Ft,350000Ft becslés.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="65" customHeight="1">
+      <x:c r="A4" s="1" t="str">
+        <x:v>KI-032</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="n">
+        <x:f>'Elemregiszter'!U33</x:f>
+        <x:v>135000</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="n">
+        <x:f>C4-B4</x:f>
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>+15000Ft:3óra többlet szerelési előirányzat×5000Ft. Falteher és szolgáltatáskeresés továbbra ellenőrzendő.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="65" customHeight="1">
+      <x:c r="A5" s="1" t="str">
+        <x:v>KI-041</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="n">
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="n">
+        <x:f>'Elemregiszter'!U42</x:f>
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="n">
+        <x:f>C5-B5</x:f>
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>+15000Ft: magas konzol/oldható elem előirányzat; mennyezeti fúrás nincs jóváhagyva.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="65" customHeight="1">
+      <x:c r="A6" s="1" t="str">
+        <x:v>KI-042</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="n">
+        <x:v>55000</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="n">
+        <x:f>'Elemregiszter'!U43</x:f>
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="n">
+        <x:f>C6-B6</x:f>
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>+10000Ft: magas szerelés/hozzáférés előirányzat; szövetkeret KI-040 változatlan.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="65" customHeight="1">
+      <x:c r="A7" s="1" t="str">
+        <x:v>KI-R10-01</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="n">
+        <x:f>'Elemregiszter'!U179</x:f>
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="n">
+        <x:f>C7-B7</x:f>
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Tervezői becslés:3×8000Ft párna+21000Ft takaró;30000–60000Ft sáv</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32169,7 +32328,7 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H31" s="19" t="str">
-        <x:v>W01 panelkompozíció és sötét tusgrafikás torony</x:v>
+        <x:v>W01:720mm torony +120mm visszahúzott sáv +4×690mm panel; összes3600mm</x:v>
       </x:c>
       <x:c r="I31" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -32181,7 +32340,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="L31" s="19" t="str">
-        <x:v>TV-01: 700×400×2330 mm; TV-03: 2600×36×2330 mm</x:v>
+        <x:v>720×400×2330 felső torony;2760×36×2330 panel</x:v>
       </x:c>
       <x:c r="M31" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -32196,7 +32355,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q31" s="20" t="n">
-        <x:v>690000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="R31" s="20" t="n">
         <x:v>0</x:v>
@@ -32209,7 +32368,7 @@
       </x:c>
       <x:c r="U31" s="21" t="n">
         <x:f>O31*Q31+SUM(R31:T31)</x:f>
-        <x:v>690000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="V31" s="19" t="str">
         <x:v>előzetes becslés</x:v>
@@ -32218,7 +32377,7 @@
         <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X31" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="Y31" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32242,14 +32401,14 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF31" s="19" t="str">
-        <x:v>R05: referencia a VISUAL_RESCUE. 450000 eredeti+160000 felület+80000 grafika/minta. Nem külön újra összegezendő.</x:v>
+        <x:v>+75500Ft becslés:0,4194m² többletfelület kb10500Ft; köztes sáv25000; szélek/alkatrész10000; új hordozó/nyomatpróba30000. Nem ajánlat.</x:v>
       </x:c>
       <x:c r="AG31" s="20" t="n">
-        <x:v>590000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="AH31" s="21" t="n">
         <x:f>O31*AG31+SUM(R31:T31)</x:f>
-        <x:v>590000</x:v>
+        <x:v>765500</x:v>
       </x:c>
       <x:c r="AI31" s="19" t="str">
         <x:v>Kézzel texturált mezők helyett sík, gyári szövethatású nyomtatott hordozó;160000 felületi felárból60000 marad. A torony és tuskompozíció változatlan. Eltérés: súrolófényben laposabb felület, nem teljes anyagazonosság; nem jóváhagyott. Nettó projektmegtakarítás 100000 Ft, bruttó költségek különbsége.</x:v>
@@ -32270,10 +32429,10 @@
         <x:v>TV-01; TV-03</x:v>
       </x:c>
       <x:c r="AO31" s="1" t="str">
-        <x:v>CP3/drawings/TV-01_CP3.pdf; CP3/drawings/TV-03_CP3.pdf</x:v>
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
       </x:c>
       <x:c r="AP31" s="1" t="str">
-        <x:v>CP3_TV-01; CP3_TV-03</x:v>
+        <x:v>R10_INK_R10_*;R10_TV01*;R10_TV02*</x:v>
       </x:c>
       <x:c r="AQ31" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
@@ -32307,11 +32466,11 @@
       </x:c>
       <x:c r="BA31" s="29" t="n">
         <x:f>ROUND(U31*AY31,0)</x:f>
-        <x:v>560000</x:v>
+        <x:v>621275</x:v>
       </x:c>
       <x:c r="BB31" s="29" t="n">
         <x:f>ROUND(U31*AZ31,0)</x:f>
-        <x:v>950000</x:v>
+        <x:v>1053949</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="72" customHeight="1">
@@ -32337,7 +32496,7 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H32" s="19" t="str">
-        <x:v>W01 alsó ötfrontos médiabútor; torony felől700+4×650</x:v>
+        <x:v>W01 alsó bútor,5 működő front és120mm süllyesztett szervizbetét</x:v>
       </x:c>
       <x:c r="I32" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -32349,7 +32508,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="L32" s="19" t="str">
-        <x:v>TV-02: 3300×400×400 mm</x:v>
+        <x:v>3600×400×400mm;720+120+4×690</x:v>
       </x:c>
       <x:c r="M32" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -32364,7 +32523,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q32" s="20" t="n">
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="R32" s="20" t="n">
         <x:v>0</x:v>
@@ -32377,7 +32536,7 @@
       </x:c>
       <x:c r="U32" s="21" t="n">
         <x:f>O32*Q32+SUM(R32:T32)</x:f>
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="V32" s="19" t="str">
         <x:v>előzetes becslés</x:v>
@@ -32386,7 +32545,7 @@
         <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
       </x:c>
       <x:c r="X32" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="Y32" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32410,14 +32569,14 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF32" s="19" t="str">
-        <x:v>260000 eredeti+60000 front/illesztés felár. Belső fiókelhagyásból nem számolunk fiktív megtakarítást.</x:v>
+        <x:v>+30000Ft:300mm többlet korpusz/top/front, régi320000×3600/3300≈349091Ft,350000Ft becslés.</x:v>
       </x:c>
       <x:c r="AG32" s="20" t="n">
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="AH32" s="21" t="n">
         <x:f>O32*AG32+SUM(R32:T32)</x:f>
-        <x:v>320000</x:v>
+        <x:v>350000</x:v>
       </x:c>
       <x:c r="AI32" s="19" t="str">
         <x:v>R05 főváltozat tartalma; korábbi fiók-/aszimmetria-elhagyás nincs automatikusan kiválasztva.</x:v>
@@ -32438,10 +32597,10 @@
         <x:v>TV-02</x:v>
       </x:c>
       <x:c r="AO32" s="1" t="str">
-        <x:v>CP3/drawings/TV-02_CP3.pdf</x:v>
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
       </x:c>
       <x:c r="AP32" s="1" t="str">
-        <x:v>CP3_TV-02</x:v>
+        <x:v>R10_TV03*</x:v>
       </x:c>
       <x:c r="AQ32" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
@@ -32475,11 +32634,11 @@
       </x:c>
       <x:c r="BA32" s="29" t="n">
         <x:f>ROUND(U32*AY32,0)</x:f>
-        <x:v>256000</x:v>
+        <x:v>280000</x:v>
       </x:c>
       <x:c r="BB32" s="29" t="n">
         <x:f>ROUND(U32*AZ32,0)</x:f>
-        <x:v>448000</x:v>
+        <x:v>490000</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="72" customHeight="1">
@@ -32505,7 +32664,7 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H33" s="19" t="str">
-        <x:v>W01 rögzítés, szerviznyílás, szerelés</x:v>
+        <x:v>W01 rögzítés, szerviz és köztes sáv szerelése</x:v>
       </x:c>
       <x:c r="I33" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -32517,7 +32676,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="L33" s="19" t="str">
-        <x:v>TV-01: 700×400×2330 mm; TV-02: 3300×400×400 mm; TV-03: 2600×36×2330 mm</x:v>
+        <x:v>R10 TV-01/02/03; tervi4m fal</x:v>
       </x:c>
       <x:c r="M33" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -32532,7 +32691,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q33" s="20" t="n">
-        <x:v>120000</x:v>
+        <x:v>135000</x:v>
       </x:c>
       <x:c r="R33" s="20" t="n">
         <x:v>0</x:v>
@@ -32545,7 +32704,7 @@
       </x:c>
       <x:c r="U33" s="21" t="n">
         <x:f>O33*Q33+SUM(R33:T33)</x:f>
-        <x:v>120000</x:v>
+        <x:v>135000</x:v>
       </x:c>
       <x:c r="V33" s="19" t="str">
         <x:v>előzetes becslés</x:v>
@@ -32554,7 +32713,7 @@
         <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03a</x:v>
       </x:c>
       <x:c r="X33" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="Y33" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32578,14 +32737,14 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF33" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>+15000Ft:3óra többlet szerelési előirányzat×5000Ft. Falteher és szolgáltatáskeresés továbbra ellenőrzendő.</x:v>
       </x:c>
       <x:c r="AG33" s="20" t="n">
-        <x:v>120000</x:v>
+        <x:v>135000</x:v>
       </x:c>
       <x:c r="AH33" s="21" t="n">
         <x:f>O33*AG33+SUM(R33:T33)</x:f>
-        <x:v>120000</x:v>
+        <x:v>135000</x:v>
       </x:c>
       <x:c r="AI33" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -32606,10 +32765,10 @@
         <x:v>TV-01; TV-02; TV-03</x:v>
       </x:c>
       <x:c r="AO33" s="1" t="str">
-        <x:v>CP3/drawings/TV-01_CP3.pdf; CP3/drawings/TV-02_CP3.pdf; CP3/drawings/TV-03_CP3.pdf</x:v>
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
       </x:c>
       <x:c r="AP33" s="1" t="str">
-        <x:v>CP3_TV-01; CP3_TV-02; CP3_TV-03</x:v>
+        <x:v>R10_TV*</x:v>
       </x:c>
       <x:c r="AQ33" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
@@ -32643,11 +32802,11 @@
       </x:c>
       <x:c r="BA33" s="29" t="n">
         <x:f>ROUND(U33*AY33,0)</x:f>
-        <x:v>102000</x:v>
+        <x:v>114750</x:v>
       </x:c>
       <x:c r="BB33" s="29" t="n">
         <x:f>ROUND(U33*AZ33,0)</x:f>
-        <x:v>156000</x:v>
+        <x:v>175500</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
@@ -34017,7 +34176,7 @@
         <x:v>Textil</x:v>
       </x:c>
       <x:c r="H42" s="19" t="str">
-        <x:v>Fali sín, konzolok, végzárók és rögzítés</x:v>
+        <x:v>Magas fali sín, konzolok és oldható szervizrögzítés</x:v>
       </x:c>
       <x:c r="I42" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -34029,7 +34188,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="L42" s="19" t="str">
-        <x:v>UNKNOWN – felmérés/gyári adat kell</x:v>
+        <x:v>4500mm sín; z2840mm javaslat</x:v>
       </x:c>
       <x:c r="M42" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -34044,7 +34203,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q42" s="20" t="n">
-        <x:v>65000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="R42" s="20" t="n">
         <x:v>0</x:v>
@@ -34057,7 +34216,7 @@
       </x:c>
       <x:c r="U42" s="21" t="n">
         <x:f>O42*Q42+SUM(R42:T42)</x:f>
-        <x:v>65000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="V42" s="19" t="str">
         <x:v>előzetes becslés</x:v>
@@ -34066,7 +34225,7 @@
         <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03f</x:v>
       </x:c>
       <x:c r="X42" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="Y42" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -34090,14 +34249,14 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF42" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>+15000Ft: magas konzol/oldható elem előirányzat; mennyezeti fúrás nincs jóváhagyva.</x:v>
       </x:c>
       <x:c r="AG42" s="20" t="n">
-        <x:v>65000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="AH42" s="21" t="n">
         <x:f>O42*AG42+SUM(R42:T42)</x:f>
-        <x:v>65000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="AI42" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -34118,10 +34277,10 @@
         <x:v>KI-041</x:v>
       </x:c>
       <x:c r="AO42" s="1" t="str">
-        <x:v>drawings/P-01_alaprajz.pdf</x:v>
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
       </x:c>
       <x:c r="AP42" s="1" t="str">
-        <x:v>NINCS MODELL / nem térbeli költségsor; szakági kapcsolat igazolandó</x:v>
+        <x:v>R09_curtain_track*</x:v>
       </x:c>
       <x:c r="AQ42" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
@@ -34155,11 +34314,11 @@
       </x:c>
       <x:c r="BA42" s="29" t="n">
         <x:f>ROUND(U42*AY42,0)</x:f>
-        <x:v>55250</x:v>
+        <x:v>68000</x:v>
       </x:c>
       <x:c r="BB42" s="29" t="n">
         <x:f>ROUND(U42*AZ42,0)</x:f>
-        <x:v>84500</x:v>
+        <x:v>104000</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="72" customHeight="1">
@@ -34185,7 +34344,7 @@
         <x:v>Textil</x:v>
       </x:c>
       <x:c r="H43" s="19" t="str">
-        <x:v>Méretre varrás és függönyszerelés</x:v>
+        <x:v>Méretre varrás és magas függönyszerelés</x:v>
       </x:c>
       <x:c r="I43" s="19" t="str">
         <x:v>UNKNOWN</x:v>
@@ -34197,7 +34356,7 @@
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="L43" s="19" t="str">
-        <x:v>UNKNOWN – felmérés/gyári adat kell</x:v>
+        <x:v>Textil felső él2810mm; alsó él15mm; hossz2795mm tervezett, helyszíni felmérésre vár.</x:v>
       </x:c>
       <x:c r="M43" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -34212,7 +34371,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q43" s="20" t="n">
-        <x:v>55000</x:v>
+        <x:v>65000</x:v>
       </x:c>
       <x:c r="R43" s="20" t="n">
         <x:v>0</x:v>
@@ -34225,7 +34384,7 @@
       </x:c>
       <x:c r="U43" s="21" t="n">
         <x:f>O43*Q43+SUM(R43:T43)</x:f>
-        <x:v>55000</x:v>
+        <x:v>65000</x:v>
       </x:c>
       <x:c r="V43" s="19" t="str">
         <x:v>előzetes becslés</x:v>
@@ -34234,7 +34393,7 @@
         <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03f</x:v>
       </x:c>
       <x:c r="X43" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="Y43" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -34258,14 +34417,14 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF43" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>+10000Ft: magas szerelés/hozzáférés előirányzat; szövetkeret KI-040 változatlan.</x:v>
       </x:c>
       <x:c r="AG43" s="20" t="n">
-        <x:v>55000</x:v>
+        <x:v>65000</x:v>
       </x:c>
       <x:c r="AH43" s="21" t="n">
         <x:f>O43*AG43+SUM(R43:T43)</x:f>
-        <x:v>55000</x:v>
+        <x:v>65000</x:v>
       </x:c>
       <x:c r="AI43" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -34286,10 +34445,10 @@
         <x:v>KI-042</x:v>
       </x:c>
       <x:c r="AO43" s="1" t="str">
-        <x:v>drawings/P-01_alaprajz.pdf</x:v>
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
       </x:c>
       <x:c r="AP43" s="1" t="str">
-        <x:v>NINCS MODELL / nem térbeli költségsor; szakági kapcsolat igazolandó</x:v>
+        <x:v>R09_gathered_sheer*</x:v>
       </x:c>
       <x:c r="AQ43" s="1" t="str">
         <x:v>késztermék / szakági munka</x:v>
@@ -34323,11 +34482,11 @@
       </x:c>
       <x:c r="BA43" s="29" t="n">
         <x:f>ROUND(U43*AY43,0)</x:f>
-        <x:v>46750</x:v>
+        <x:v>55250</x:v>
       </x:c>
       <x:c r="BB43" s="29" t="n">
         <x:f>ROUND(U43*AZ43,0)</x:f>
-        <x:v>71500</x:v>
+        <x:v>84500</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="72" customHeight="1">
@@ -46289,7 +46448,7 @@
         <x:v>https://files.hafele.co.uk/catalogfiles/www/25-1010.pdf</x:v>
       </x:c>
       <x:c r="L115" s="19" t="str">
-        <x:v>Felső2,60m + függőleges2,33m + alsó3,30m; összes8,23m,10m rendelés</x:v>
+        <x:v>Felső2,76m + függőleges2,33m + alsó3,60m=8,69m;10m rendelési keret</x:v>
       </x:c>
       <x:c r="M115" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
@@ -56874,6 +57033,174 @@
       <x:c r="BB178" s="29" t="n">
         <x:f>ROUND(U178*AZ178,0)</x:f>
         <x:v>180000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="12" t="str">
+        <x:v>A-902</x:v>
+      </x:c>
+      <x:c r="B179" s="12" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="C179" s="12" t="str">
+        <x:v>KI-R10-01</x:v>
+      </x:c>
+      <x:c r="D179" s="12" t="str">
+        <x:v>Cam12 v1; Cam02 v1</x:v>
+      </x:c>
+      <x:c r="E179" s="12" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F179" s="12" t="str">
+        <x:v>STÍLUS</x:v>
+      </x:c>
+      <x:c r="G179" s="12" t="str">
+        <x:v>Textil</x:v>
+      </x:c>
+      <x:c r="H179" s="19" t="str">
+        <x:v>3 díszpárna és1 takaró, külön beszerzés</x:v>
+      </x:c>
+      <x:c r="I179" s="19" t="str">
+        <x:v>választandó</x:v>
+      </x:c>
+      <x:c r="J179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="K179" s="19" t="str">
+        <x:v>UNKNOWN</x:v>
+      </x:c>
+      <x:c r="L179" s="19" t="str">
+        <x:v>3×kb43×43cm;1 takaró, méret/termék egyeztetendő</x:v>
+      </x:c>
+      <x:c r="M179" s="19" t="str">
+        <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
+      </x:c>
+      <x:c r="N179" s="19" t="str">
+        <x:v>PENDING – műszaki specifikáció szerint</x:v>
+      </x:c>
+      <x:c r="O179" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P179" s="19" t="str">
+        <x:v>csomag</x:v>
+      </x:c>
+      <x:c r="Q179" s="20" t="n">
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="R179" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S179" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T179" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U179" s="21" t="n">
+        <x:f>O179*Q179+SUM(R179:T179)</x:f>
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="V179" s="19" t="str">
+        <x:v>előzetes becslés</x:v>
+      </x:c>
+      <x:c r="W179" s="19" t="str">
+        <x:v>Tervezői becslés:3×8000Ft párna+21000Ft takaró;30000–60000Ft sáv</x:v>
+      </x:c>
+      <x:c r="X179" s="19" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c r="Y179" s="19" t="str">
+        <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
+      </x:c>
+      <x:c r="Z179" s="19" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="AA179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AB179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AC179" s="19" t="str">
+        <x:v>nem megrendelt</x:v>
+      </x:c>
+      <x:c r="AD179" s="19" t="str">
+        <x:v>Beszerzési felelős / Péter</x:v>
+      </x:c>
+      <x:c r="AE179" s="19" t="str">
+        <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
+      </x:c>
+      <x:c r="AF179" s="19" t="str">
+        <x:v>R09 külön deltája most egyszer átvezetve; nem a Lennon gyári tartozéka.</x:v>
+      </x:c>
+      <x:c r="AG179" s="20" t="n">
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="AH179" s="21" t="n">
+        <x:f>O179*AG179+SUM(R179:T179)</x:f>
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="AI179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AJ179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AK179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AL179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AM179" s="19" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="AN179" s="1" t="str">
+        <x:v>KI-135</x:v>
+      </x:c>
+      <x:c r="AO179" s="1" t="str">
+        <x:v>R10/drawings/W01_R10.pdf</x:v>
+      </x:c>
+      <x:c r="AP179" s="1" t="str">
+        <x:v>R09_cushion_*, R09_grey_throw</x:v>
+      </x:c>
+      <x:c r="AQ179" s="1" t="str">
+        <x:v>késztermék / szakági munka</x:v>
+      </x:c>
+      <x:c r="AR179" s="1" t="str">
+        <x:v>felmérés/gyártói rajz szükséges</x:v>
+      </x:c>
+      <x:c r="AS179" s="1" t="str">
+        <x:v>HUF</x:v>
+      </x:c>
+      <x:c r="AT179" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU179" s="1" t="str">
+        <x:v>nincs visszaigazolt ajánlati érvényesség</x:v>
+      </x:c>
+      <x:c r="AV179" s="1" t="str">
+        <x:v>KI-151 központi keret; daruzás KI-137</x:v>
+      </x:c>
+      <x:c r="AW179" s="1" t="str">
+        <x:v>KI-014 asztalos / KI-106 villamos / KI-026 és KI-096 víz / KI-127 fal</x:v>
+      </x:c>
+      <x:c r="AX179" s="1" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="AY179" s="1" t="n">
+        <x:v>0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="AZ179" s="1" t="n">
+        <x:v>1.3333333333333333</x:v>
+      </x:c>
+      <x:c r="BA179" s="29" t="n">
+        <x:f>ROUND(U179*AY179,0)</x:f>
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="BB179" s="29" t="n">
+        <x:f>ROUND(U179*AZ179,0)</x:f>
+        <x:v>60000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -56887,7 +57214,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1a3955fcbed43fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf05aa4e9d6a24906"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -56939,11 +57266,11 @@
         <x:v>400000</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A2)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A2)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="E2" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A2)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A2)</x:f>
         <x:v>420000</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
@@ -56965,11 +57292,11 @@
         <x:v>1100000</x:v>
       </x:c>
       <x:c r="D3" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A3)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A3)</x:f>
         <x:v>1285000</x:v>
       </x:c>
       <x:c r="E3" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A3)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A3)</x:f>
         <x:v>1285000</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
@@ -56991,11 +57318,11 @@
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A4)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A4)</x:f>
         <x:v>252990</x:v>
       </x:c>
       <x:c r="E4" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A4)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A4)</x:f>
         <x:v>252990</x:v>
       </x:c>
       <x:c r="F4" s="18" t="n">
@@ -57017,11 +57344,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D5" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A5)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A5)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="E5" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A5)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A5)</x:f>
         <x:v>1179980</x:v>
       </x:c>
       <x:c r="F5" s="18" t="n">
@@ -57043,11 +57370,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D6" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A6)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A6)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="E6" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A6)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A6)</x:f>
         <x:v>1157380</x:v>
       </x:c>
       <x:c r="F6" s="18" t="n">
@@ -57069,11 +57396,11 @@
         <x:v>500000</x:v>
       </x:c>
       <x:c r="D7" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A7)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A7)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="E7" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A7)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A7)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="F7" s="18" t="n">
@@ -57095,11 +57422,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D8" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A8)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A8)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="E8" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A8)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A8)</x:f>
         <x:v>485000</x:v>
       </x:c>
       <x:c r="F8" s="18" t="n">
@@ -57121,11 +57448,11 @@
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="D9" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A9)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A9)</x:f>
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A9)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A9)</x:f>
         <x:v>1700000</x:v>
       </x:c>
       <x:c r="F9" s="18" t="n">
@@ -57147,11 +57474,11 @@
         <x:v>300000</x:v>
       </x:c>
       <x:c r="D10" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A10)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A10)</x:f>
         <x:v>300000</x:v>
       </x:c>
       <x:c r="E10" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A10)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A10)</x:f>
         <x:v>300000</x:v>
       </x:c>
       <x:c r="F10" s="18" t="n">
@@ -57173,11 +57500,11 @@
         <x:v>600000</x:v>
       </x:c>
       <x:c r="D11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A11)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A11)</x:f>
         <x:v>600000</x:v>
       </x:c>
       <x:c r="E11" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A11)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A11)</x:f>
         <x:v>600000</x:v>
       </x:c>
       <x:c r="F11" s="18" t="n">
@@ -57199,11 +57526,11 @@
         <x:v>550000</x:v>
       </x:c>
       <x:c r="D12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A12)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A12)</x:f>
         <x:v>550000</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A12)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A12)</x:f>
         <x:v>550000</x:v>
       </x:c>
       <x:c r="F12" s="18" t="n">
@@ -57225,11 +57552,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D13" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A13)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A13)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="E13" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A13)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A13)</x:f>
         <x:v>590000</x:v>
       </x:c>
       <x:c r="F13" s="18" t="n">
@@ -57251,11 +57578,11 @@
         <x:v>450000</x:v>
       </x:c>
       <x:c r="D14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A14)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A14)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="E14" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A14)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A14)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="F14" s="18" t="n">
@@ -57277,11 +57604,11 @@
         <x:v>1189000</x:v>
       </x:c>
       <x:c r="D15" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A15)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A15)</x:f>
         <x:v>1450000</x:v>
       </x:c>
       <x:c r="E15" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A15)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A15)</x:f>
         <x:v>1450000</x:v>
       </x:c>
       <x:c r="F15" s="18" t="n">
@@ -57303,16 +57630,16 @@
         <x:v>861000</x:v>
       </x:c>
       <x:c r="D16" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A16)</x:f>
-        <x:v>1450000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A16)</x:f>
+        <x:v>1570500</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A16)</x:f>
-        <x:v>1350000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A16)</x:f>
+        <x:v>1570500</x:v>
       </x:c>
       <x:c r="F16" s="18" t="n">
         <x:f>E16-C16</x:f>
-        <x:v>489000</x:v>
+        <x:v>709500</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
         <x:v>W01 teljes panelkompozíció és tusgrafikás torony; W01 alsó négyfrontos médiabútor; W01 rögzítés, szerviznyílás, szerelés; TV készülék 65 col célkategória; Teherhordó TV-konzol; HDMI, hálózat, kábelszervezés, audióigény előirányzat</x:v>
@@ -57329,11 +57656,11 @@
         <x:v>800000</x:v>
       </x:c>
       <x:c r="D17" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A17)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A17)</x:f>
         <x:v>800000</x:v>
       </x:c>
       <x:c r="E17" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A17)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A17)</x:f>
         <x:v>800000</x:v>
       </x:c>
       <x:c r="F17" s="18" t="n">
@@ -57355,11 +57682,11 @@
         <x:v>220000</x:v>
       </x:c>
       <x:c r="D18" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A18)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A18)</x:f>
         <x:v>160000</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A18)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A18)</x:f>
         <x:v>160000</x:v>
       </x:c>
       <x:c r="F18" s="18" t="n">
@@ -57381,11 +57708,11 @@
         <x:v>760000</x:v>
       </x:c>
       <x:c r="D19" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A19)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A19)</x:f>
         <x:v>711070</x:v>
       </x:c>
       <x:c r="E19" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A19)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A19)</x:f>
         <x:v>711070</x:v>
       </x:c>
       <x:c r="F19" s="18" t="n">
@@ -57407,11 +57734,11 @@
         <x:v>200000</x:v>
       </x:c>
       <x:c r="D20" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A20)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A20)</x:f>
         <x:v>200000</x:v>
       </x:c>
       <x:c r="E20" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A20)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A20)</x:f>
         <x:v>200000</x:v>
       </x:c>
       <x:c r="F20" s="18" t="n">
@@ -57433,16 +57760,16 @@
         <x:v>260000</x:v>
       </x:c>
       <x:c r="D21" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A21)</x:f>
-        <x:v>280000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A21)</x:f>
+        <x:v>305000</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A21)</x:f>
-        <x:v>280000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A21)</x:f>
+        <x:v>305000</x:v>
       </x:c>
       <x:c r="F21" s="18" t="n">
         <x:f>E21-C21</x:f>
-        <x:v>20000</x:v>
+        <x:v>45000</x:v>
       </x:c>
       <x:c r="G21" s="19" t="str">
         <x:v>Nappali fényáteresztő és sötétítő szövet; Fali sín, konzolok, végzárók és rögzítés; Méretre varrás és függönyszerelés</x:v>
@@ -57459,11 +57786,11 @@
         <x:v>550000</x:v>
       </x:c>
       <x:c r="D22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A22)</x:f>
         <x:v>499900</x:v>
       </x:c>
       <x:c r="E22" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A22)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A22)</x:f>
         <x:v>499900</x:v>
       </x:c>
       <x:c r="F22" s="18" t="n">
@@ -57485,11 +57812,11 @@
         <x:v>353000</x:v>
       </x:c>
       <x:c r="D23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A23)</x:f>
         <x:v>355000</x:v>
       </x:c>
       <x:c r="E23" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A23)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A23)</x:f>
         <x:v>355000</x:v>
       </x:c>
       <x:c r="F23" s="18" t="n">
@@ -57511,11 +57838,11 @@
         <x:v>820000</x:v>
       </x:c>
       <x:c r="D24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A24)</x:f>
         <x:v>1996000</x:v>
       </x:c>
       <x:c r="E24" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A24)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A24)</x:f>
         <x:v>1996000</x:v>
       </x:c>
       <x:c r="F24" s="18" t="n">
@@ -57537,11 +57864,11 @@
         <x:v>380000</x:v>
       </x:c>
       <x:c r="D25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A25)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="E25" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A25)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A25)</x:f>
         <x:v>480000</x:v>
       </x:c>
       <x:c r="F25" s="18" t="n">
@@ -57563,11 +57890,11 @@
         <x:v>820000</x:v>
       </x:c>
       <x:c r="D26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A26)</x:f>
         <x:v>1085000</x:v>
       </x:c>
       <x:c r="E26" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A26)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A26)</x:f>
         <x:v>1085000</x:v>
       </x:c>
       <x:c r="F26" s="18" t="n">
@@ -57589,11 +57916,11 @@
         <x:v>1400000</x:v>
       </x:c>
       <x:c r="D27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A27)</x:f>
         <x:v>2060360</x:v>
       </x:c>
       <x:c r="E27" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A27)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A27)</x:f>
         <x:v>2060360</x:v>
       </x:c>
       <x:c r="F27" s="18" t="n">
@@ -57615,11 +57942,11 @@
         <x:v>336000</x:v>
       </x:c>
       <x:c r="D28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A28)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="E28" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A28)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A28)</x:f>
         <x:v>405000</x:v>
       </x:c>
       <x:c r="F28" s="18" t="n">
@@ -57641,16 +57968,16 @@
         <x:v>262000</x:v>
       </x:c>
       <x:c r="D29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A29)</x:f>
-        <x:v>551000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A29)</x:f>
+        <x:v>596000</x:v>
       </x:c>
       <x:c r="E29" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A29)</x:f>
-        <x:v>503000</x:v>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A29)</x:f>
+        <x:v>548000</x:v>
       </x:c>
       <x:c r="F29" s="18" t="n">
         <x:f>E29-C29</x:f>
-        <x:v>241000</x:v>
+        <x:v>286000</x:v>
       </x:c>
       <x:c r="G29" s="19" t="str">
         <x:v>W02 eredeti tusgrafika előállítása és nyomdai előkészítése; W02 textilnyomat 150×220 célméret; W02 vékony keret, szállítás és rögzítés; Nappali párnák és takaró; Kerámiák, művészeti könyvek és kisebb növények</x:v>
@@ -57667,11 +57994,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$178,'Elemregiszter'!$E$2:$E$178,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A30)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="E30" s="18" t="n">
-        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$178,'Elemregiszter'!$E$2:$E$178,A30)</x:f>
+        <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A30)</x:f>
         <x:v>510000</x:v>
       </x:c>
       <x:c r="F30" s="18" t="n">
@@ -57696,15 +58023,15 @@
       </x:c>
       <x:c r="D31" s="18" t="n">
         <x:f>SUM(D2:D30)</x:f>
-        <x:v>22503680</x:v>
+        <x:v>22694180</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
         <x:f>SUM(E2:E30)</x:f>
-        <x:v>22355680</x:v>
+        <x:v>22646180</x:v>
       </x:c>
       <x:c r="F31" s="18" t="n">
         <x:f>SUM(F2:F30)</x:f>
-        <x:v>4744680</x:v>
+        <x:v>5035180</x:v>
       </x:c>
       <x:c r="G31" s="19"/>
     </x:row>

</xml_diff>

<commit_message>
R16: update TV wall with 200mm bronze infill, source-traced ink, six push-to-open soft-close drawer designs and eight opening-light circuits; synchronize CAD, drawings, labels and live budget
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/outputs/A902_Kyoto_Ink_elo_regiszter.xlsx
@@ -2,31 +2,32 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R824f5e37e7314c1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="Re9de161a947c4ab7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="R9dceecd1562548d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="R16cf21137f82446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="R04d67890da524bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="Rbc81d6d2a8a34243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="R6e44304fd72a4ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="Rf718dd1e79b64ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="R048b2710971d4a6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="R92812f3040a14b8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="R89f0fb5c34cc4b4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="R88e5401dc66249c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="R30a183406d444737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="Rf5ba364675f3465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="R5f757a4fff364951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R3d74062258c94d87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="R75627b8a59e44fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="Rebd0add04ec04da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="R121bb85634de46fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="R977ff9c348a74821"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R37d48707329c4b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R4a47cf488fc248e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="Re05e8dfc69914f1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 változások" sheetId="24" r:id="R51c0e764b322439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R10 változások" sheetId="25" r:id="R44cb221dc96e4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiemelt termékek" sheetId="1" r:id="R586ba43f0c804e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Összesítő" sheetId="2" r:id="R67bec8bc062b487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elemregiszter" sheetId="3" r:id="Rffa9dcaf285344ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline egyeztetés" sheetId="4" r:id="Rc0853b2667d14fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lefedettség" sheetId="5" r:id="R992e1b243a9b4889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Világítás" sheetId="6" r:id="Rf3d3341fa3f648f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felületi mennyiségek" sheetId="7" r:id="R3226f27760da456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textilmennyiségek" sheetId="8" r:id="R546eb52363134e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nyitott döntések" sheetId="9" r:id="R21639e3338334f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ütemterv" sheetId="10" r:id="R6b98bd611769484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="További termékek" sheetId="11" r:id="R5ec1ab154bd54936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP1a eltérések" sheetId="12" r:id="R35d6ee8a12b44c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vizuális eltérések" sheetId="13" r:id="R56198283dfd24fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Előzetes szabáslista" sheetId="14" r:id="Ra3c07da3f9b9492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05.2 alternatíva" sheetId="15" r:id="Rf0a396387a0d46a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 rekeszek" sheetId="16" r:id="R2cdae1618c0f4faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 belső fény" sheetId="17" r:id="R42c1341125e14496"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 tápegységek" sheetId="18" r:id="Rd5782aee909845f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 vasalat" sheetId="19" r:id="R0dbd1474b9774dc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP3 eltérések" sheetId="20" r:id="Rc19e4172d37f42c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 anyagok" sheetId="21" r:id="R39d4d0907b264c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 változások" sheetId="22" r:id="R467977fc701148b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 kapacitás" sheetId="23" r:id="Reebcd432d52d4a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 változások" sheetId="24" r:id="Rfa0463b0dc404cac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R10 változások" sheetId="25" r:id="Rf63bba298bf94da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R16 változások" sheetId="26" r:id="R8fefbf4edf5d46af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,7 +198,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -374,6 +375,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2886,11 +2890,11 @@
       </x:c>
       <x:c r="D31" s="19" t="n">
         <x:f>'Elemregiszter'!U31</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="E31" s="19" t="n">
         <x:f>D31-C31</x:f>
-        <x:v>455500</x:v>
+        <x:v>625500</x:v>
       </x:c>
       <x:c r="F31" s="19" t="str">
         <x:v>W01 V3.3 panelmező, grafikus torony: nagyobb folytonos grafika; 3600×2880 tervezési befoglaló</x:v>
@@ -2908,11 +2912,11 @@
       </x:c>
       <x:c r="D32" s="19" t="n">
         <x:f>'Elemregiszter'!U32</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="E32" s="19" t="n">
         <x:f>D32-C32</x:f>
-        <x:v>140000</x:v>
+        <x:v>775000</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str">
         <x:v>W01 V3.3 folytonos alsó tároló: 3300×400×400, 5 front</x:v>
@@ -2930,11 +2934,11 @@
       </x:c>
       <x:c r="D33" s="19" t="n">
         <x:f>'Elemregiszter'!U33</x:f>
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="E33" s="19" t="n">
         <x:f>D33-C33</x:f>
-        <x:v>15000</x:v>
+        <x:v>384800</x:v>
       </x:c>
       <x:c r="F33" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -2974,11 +2978,11 @@
       </x:c>
       <x:c r="D35" s="19" t="n">
         <x:f>'Elemregiszter'!U35</x:f>
-        <x:v>30000</x:v>
+        <x:v>32000</x:v>
       </x:c>
       <x:c r="E35" s="19" t="n">
         <x:f>D35-C35</x:f>
-        <x:v>0</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="F35" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -4734,11 +4738,11 @@
       </x:c>
       <x:c r="D115" s="19" t="n">
         <x:f>'Elemregiszter'!U115</x:f>
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="E115" s="19" t="n">
         <x:f>D115-C115</x:f>
-        <x:v>0</x:v>
+        <x:v>362000</x:v>
       </x:c>
       <x:c r="F115" s="19" t="str">
         <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
@@ -19704,7 +19708,7 @@
       </x:c>
       <x:c r="B7" s="18" t="n">
         <x:f>SUM('Elemregiszter'!U2:U179)</x:f>
-        <x:v>24673390</x:v>
+        <x:v>26212190</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
         <x:v>R10:3600mm médiafal,120mm sáv, magas függöny, külön textilek. Becslések, nem jóváhagyott többletkeret.</x:v>
@@ -19716,7 +19720,7 @@
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f>SUM('Elemregiszter'!AH2:AH179)</x:f>
-        <x:v>24520390</x:v>
+        <x:v>26059190</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
         <x:v>Összehasonlítható takarékos változat:253000Ft dokumentált megtakarítás;18M továbbra sem igazolt.</x:v>
@@ -19728,7 +19732,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>B7-B5</x:f>
-        <x:v>6673390</x:v>
+        <x:v>8212190</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19740,7 +19744,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>B8-B5</x:f>
-        <x:v>6520390</x:v>
+        <x:v>8059190</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>Pozitív = túllépés</x:v>
@@ -19776,7 +19780,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>B7-B11-B12</x:f>
-        <x:v>22530950</x:v>
+        <x:v>24069750</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>Minden nem igazolt ár</x:v>
@@ -19899,11 +19903,11 @@
       </x:c>
       <x:c r="B25" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$B$2:$B$179,A25)</x:f>
-        <x:v>3932690</x:v>
+        <x:v>5471490</x:v>
       </x:c>
       <x:c r="C25" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$B$2:$B$179,A25)</x:f>
-        <x:v>3884690</x:v>
+        <x:v>5423490</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
@@ -20167,11 +20171,11 @@
       </x:c>
       <x:c r="B47" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A47)</x:f>
-        <x:v>6336500</x:v>
+        <x:v>7511300</x:v>
       </x:c>
       <x:c r="C47" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A47)</x:f>
-        <x:v>6336500</x:v>
+        <x:v>7511300</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="30" customHeight="1">
@@ -20219,11 +20223,11 @@
       </x:c>
       <x:c r="B51" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A51)</x:f>
-        <x:v>680000</x:v>
+        <x:v>682000</x:v>
       </x:c>
       <x:c r="C51" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A51)</x:f>
-        <x:v>680000</x:v>
+        <x:v>682000</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="30" customHeight="1">
@@ -20258,11 +20262,11 @@
       </x:c>
       <x:c r="B54" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$G$2:$G$179,A54)</x:f>
-        <x:v>2200360</x:v>
+        <x:v>2562360</x:v>
       </x:c>
       <x:c r="C54" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$G$2:$G$179,A54)</x:f>
-        <x:v>2200360</x:v>
+        <x:v>2562360</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="30" customHeight="1">
@@ -20370,11 +20374,11 @@
       </x:c>
       <x:c r="B64" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$F$2:$F$179,A64)</x:f>
-        <x:v>13183830</x:v>
+        <x:v>14722630</x:v>
       </x:c>
       <x:c r="C64" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$F$2:$F$179,A64)</x:f>
-        <x:v>13135830</x:v>
+        <x:v>14674630</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="30" customHeight="1">
@@ -20404,11 +20408,11 @@
       </x:c>
       <x:c r="B68" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$AC$2:$AC$179,A68)</x:f>
-        <x:v>22694180</x:v>
+        <x:v>24232980</x:v>
       </x:c>
       <x:c r="C68" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$AC$2:$AC$179,A68)</x:f>
-        <x:v>22646180</x:v>
+        <x:v>24184980</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -20440,7 +20444,7 @@
       </x:c>
       <x:c r="B74" s="30" t="n">
         <x:f>SUM('Elemregiszter'!BA2:BA179)</x:f>
-        <x:v>20990870</x:v>
+        <x:v>22260571</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>Sorok alsó feltételezéseinek összege</x:v>
@@ -20452,7 +20456,7 @@
       </x:c>
       <x:c r="B75" s="30" t="n">
         <x:f>SUM('Elemregiszter'!BB2:BB179)</x:f>
-        <x:v>33210947</x:v>
+        <x:v>35287945</x:v>
       </x:c>
       <x:c r="C75" t="str">
         <x:v>Sorok felső feltételezéseinek összege</x:v>
@@ -20546,7 +20550,7 @@
       </x:c>
       <x:c r="B84" s="30" t="n">
         <x:f>B7-B83</x:f>
-        <x:v>24338400</x:v>
+        <x:v>25877200</x:v>
       </x:c>
       <x:c r="C84" t="str">
         <x:v>Nem automatikusan kiválasztott megtakarítás</x:v>
@@ -24000,15 +24004,15 @@
       </x:c>
       <x:c r="C2" s="55" t="n">
         <x:f>'Elemregiszter'!U31</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="D2" s="55" t="n">
         <x:f>C2-B2</x:f>
-        <x:v>315500</x:v>
+        <x:v>485500</x:v>
       </x:c>
       <x:c r="E2" s="55" t="n">
         <x:f>'Elemregiszter'!AH31</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="F2" s="55" t="n">
         <x:f>C2-E2</x:f>
@@ -24027,15 +24031,15 @@
       </x:c>
       <x:c r="C3" s="55" t="n">
         <x:f>'Elemregiszter'!U32</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="D3" s="55" t="n">
         <x:f>C3-B3</x:f>
-        <x:v>90000</x:v>
+        <x:v>725000</x:v>
       </x:c>
       <x:c r="E3" s="55" t="n">
         <x:f>'Elemregiszter'!AH32</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="F3" s="55" t="n">
         <x:f>C3-E3</x:f>
@@ -24297,15 +24301,15 @@
       </x:c>
       <x:c r="C13" s="55" t="n">
         <x:f>'Elemregiszter'!U115</x:f>
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="D13" s="55" t="n">
         <x:f>C13-B13</x:f>
-        <x:v>0</x:v>
+        <x:v>362000</x:v>
       </x:c>
       <x:c r="E13" s="55" t="n">
         <x:f>'Elemregiszter'!AH115</x:f>
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="F13" s="55" t="n">
         <x:f>C13-E13</x:f>
@@ -27099,11 +27103,11 @@
       </x:c>
       <x:c r="C2" s="1" t="n">
         <x:f>'Elemregiszter'!U31</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="D2" s="1" t="n">
         <x:f>C2-B2</x:f>
-        <x:v>75500</x:v>
+        <x:v>245500</x:v>
       </x:c>
       <x:c r="E2" s="1" t="str">
         <x:v>+75500Ft becslés:0,4194m² többletfelület kb10500Ft; köztes sáv25000; szélek/alkatrész10000; új hordozó/nyomatpróba30000. Nem ajánlat.</x:v>
@@ -27118,11 +27122,11 @@
       </x:c>
       <x:c r="C3" s="1" t="n">
         <x:f>'Elemregiszter'!U32</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="D3" s="1" t="n">
         <x:f>C3-B3</x:f>
-        <x:v>30000</x:v>
+        <x:v>665000</x:v>
       </x:c>
       <x:c r="E3" s="1" t="str">
         <x:v>+30000Ft:300mm többlet korpusz/top/front, régi320000×3600/3300≈349091Ft,350000Ft becslés.</x:v>
@@ -27137,11 +27141,11 @@
       </x:c>
       <x:c r="C4" s="1" t="n">
         <x:f>'Elemregiszter'!U33</x:f>
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="D4" s="1" t="n">
         <x:f>C4-B4</x:f>
-        <x:v>15000</x:v>
+        <x:v>384800</x:v>
       </x:c>
       <x:c r="E4" s="1" t="str">
         <x:v>+15000Ft:3óra többlet szerelési előirányzat×5000Ft. Falteher és szolgáltatáskeresés továbbra ellenőrzendő.</x:v>
@@ -27202,6 +27206,182 @@
       </x:c>
       <x:c r="E7" s="1" t="str">
         <x:v>Tervezői becslés:3×8000Ft párna+21000Ft takaró;30000–60000Ft sáv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="65" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="52" customHeight="1">
+      <x:c r="A1" s="66" t="str">
+        <x:v>Elem</x:v>
+      </x:c>
+      <x:c r="B1" s="66" t="str">
+        <x:v>Előző Ft</x:v>
+      </x:c>
+      <x:c r="C1" s="66" t="str">
+        <x:v>Új Ft</x:v>
+      </x:c>
+      <x:c r="D1" s="66" t="str">
+        <x:v>Különbség Ft</x:v>
+      </x:c>
+      <x:c r="E1" s="66" t="str">
+        <x:v>Tartalom</x:v>
+      </x:c>
+      <x:c r="F1" s="66" t="str">
+        <x:v>Státusz</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="52" customHeight="1">
+      <x:c r="A2" s="66" t="str">
+        <x:v>KI-030</x:v>
+      </x:c>
+      <x:c r="B2" s="66" t="n">
+        <x:v>765500</x:v>
+      </x:c>
+      <x:c r="C2" s="66" t="n">
+        <x:v>935500</x:v>
+      </x:c>
+      <x:c r="D2" s="66" t="n">
+        <x:f>C2-B2</x:f>
+        <x:v>170000</x:v>
+      </x:c>
+      <x:c r="E2" s="66" t="str">
+        <x:v>720 mm torony +200 mm matt bronzbetét +4×670 mm falburkolati mező</x:v>
+      </x:c>
+      <x:c r="F2" s="66" t="str">
+        <x:v>Becslés; nincs megrendelve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="52" customHeight="1">
+      <x:c r="A3" s="66" t="str">
+        <x:v>KI-031</x:v>
+      </x:c>
+      <x:c r="B3" s="66" t="n">
+        <x:v>350000</x:v>
+      </x:c>
+      <x:c r="C3" s="66" t="n">
+        <x:v>985000</x:v>
+      </x:c>
+      <x:c r="D3" s="66" t="n">
+        <x:f>C3-B3</x:f>
+        <x:v>635000</x:v>
+      </x:c>
+      <x:c r="E3" s="66" t="str">
+        <x:v>Hat magas fiókos alsó médiafal, eltérő frontszélességekkel</x:v>
+      </x:c>
+      <x:c r="F3" s="66" t="str">
+        <x:v>Becslés; nincs megrendelve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="52" customHeight="1">
+      <x:c r="A4" s="66" t="str">
+        <x:v>KI-032</x:v>
+      </x:c>
+      <x:c r="B4" s="66" t="n">
+        <x:v>135000</x:v>
+      </x:c>
+      <x:c r="C4" s="66" t="n">
+        <x:v>504800</x:v>
+      </x:c>
+      <x:c r="D4" s="66" t="n">
+        <x:f>C4-B4</x:f>
+        <x:v>369800</x:v>
+      </x:c>
+      <x:c r="E4" s="66" t="str">
+        <x:v>W01 rögzítési és műhelyi csomag R15→R16 egyeztetve</x:v>
+      </x:c>
+      <x:c r="F4" s="66" t="str">
+        <x:v>Becslés; nincs megrendelve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>KI-034</x:v>
+      </x:c>
+      <x:c r="B5" s="66" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="C5" s="66" t="n">
+        <x:v>32000</x:v>
+      </x:c>
+      <x:c r="D5" s="66" t="n">
+        <x:f>C5-B5</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="E5" s="66" t="str">
+        <x:v>Vogel TVM3605 konzol</x:v>
+      </x:c>
+      <x:c r="F5" s="66" t="str">
+        <x:v>Becslés; nincs megrendelve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="66" t="str">
+        <x:v>KI-114</x:v>
+      </x:c>
+      <x:c r="B6" s="66" t="n">
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="C6" s="66" t="n">
+        <x:v>512000</x:v>
+      </x:c>
+      <x:c r="D6" s="66" t="n">
+        <x:f>C6-B6</x:f>
+        <x:v>362000</x:v>
+      </x:c>
+      <x:c r="E6" s="66" t="str">
+        <x:v>W01 hangulatfény +6fiók és2ajtó nyitásérzékelős belső fénye</x:v>
+      </x:c>
+      <x:c r="F6" s="66" t="str">
+        <x:v>Becslés; nincs megrendelve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>R16 frissített projektelőirányzat</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:f>'Összesítő'!B7</x:f>
+        <x:v>26212190</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Külön érintetlen tartalék</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>2000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Kereteltérés</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:f>B9-18000000</x:f>
+        <x:v>8212190</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Átfedés megjegyzés</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>A korábbi csomagárakat kiváltottuk. A további szakági csomagokkal esetleges átfedést beszállítói ajánlattal kell egyeztetni.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32316,7 +32496,7 @@
         <x:v>KI-030</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>CP3/render_handoff/manifest_CP3.json</x:v>
+        <x:v>R16_feluletek_fiokok/data/handoff_manifest.json</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
         <x:v>03a</x:v>
@@ -32328,25 +32508,25 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H31" s="19" t="str">
-        <x:v>W01:720mm torony +120mm visszahúzott sáv +4×690mm panel; összes3600mm</x:v>
+        <x:v>720 mm torony +200 mm matt bronzbetét +4×670 mm falburkolati mező</x:v>
       </x:c>
       <x:c r="I31" s="19" t="str">
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J31" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>M16-WALL / M16-BRONZE / M16-TOWER</x:v>
       </x:c>
       <x:c r="K31" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>R16_feluletek_fiokok/data/sources.json; gyártói adatok, nem kereskedői árforrás</x:v>
       </x:c>
       <x:c r="L31" s="19" t="str">
-        <x:v>720×400×2330 felső torony;2760×36×2330 panel</x:v>
+        <x:v>720+200+2680 mm; névleges teljes3600 mm</x:v>
       </x:c>
       <x:c r="M31" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N31" s="19" t="str">
-        <x:v>MAT-04</x:v>
+        <x:v>M16-WALL / M16-BRONZE / M16-TOWER</x:v>
       </x:c>
       <x:c r="O31" s="19" t="n">
         <x:v>1</x:v>
@@ -32355,7 +32535,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q31" s="20" t="n">
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="R31" s="20" t="n">
         <x:v>0</x:v>
@@ -32368,16 +32548,16 @@
       </x:c>
       <x:c r="U31" s="21" t="n">
         <x:f>O31*Q31+SUM(R31:T31)</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="V31" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W31" s="19" t="str">
-        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
+        <x:v>R16/data/cost.json és R15/data/cost_allowance.json; bruttó tervezői becslés, nem ajánlat</x:v>
       </x:c>
       <x:c r="X31" s="19" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="Y31" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32401,17 +32581,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF31" s="19" t="str">
-        <x:v>+75500Ft becslés:0,4194m² többletfelület kb10500Ft; köztes sáv25000; szélek/alkatrész10000; új hordozó/nyomatpróba30000. Nem ajánlat.</x:v>
+        <x:v>18 mm hordozó; Bely+Print jelölt; bronzbarna matt felület; látható tusgrafika vektorban.</x:v>
       </x:c>
       <x:c r="AG31" s="20" t="n">
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="AH31" s="21" t="n">
         <x:f>O31*AG31+SUM(R31:T31)</x:f>
-        <x:v>765500</x:v>
+        <x:v>935500</x:v>
       </x:c>
       <x:c r="AI31" s="19" t="str">
-        <x:v>Kézzel texturált mezők helyett sík, gyári szövethatású nyomtatott hordozó;160000 felületi felárból60000 marad. A torony és tuskompozíció változatlan. Eltérés: súrolófényben laposabb felület, nem teljes anyagazonosság; nem jóváhagyott. Nettó projektmegtakarítás 100000 Ft, bruttó költségek különbsége.</x:v>
+        <x:v>R16 főtartalom. Ugyanez az előirányzat; új önálló gazdaságos változat nincs igazolva.</x:v>
       </x:c>
       <x:c r="AJ31" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -32429,16 +32609,16 @@
         <x:v>TV-01; TV-03</x:v>
       </x:c>
       <x:c r="AO31" s="1" t="str">
-        <x:v>R10/drawings/W01_R10.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_asztalos_tervcsomag.pdf</x:v>
       </x:c>
       <x:c r="AP31" s="1" t="str">
-        <x:v>R10_INK_R10_*;R10_TV01*;R10_TV02*</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_koordinacio.blend; data/parts.json</x:v>
       </x:c>
       <x:c r="AQ31" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
       </x:c>
       <x:c r="AR31" s="1" t="str">
-        <x:v>R02 méretezett ajánlati terv; nem helyszíni méret</x:v>
+        <x:v>Névleges CAD-méret; nem felmérés. Minta, fal és műhelypróba nyitott.</x:v>
       </x:c>
       <x:c r="AS31" s="1" t="str">
         <x:v>HUF</x:v>
@@ -32466,11 +32646,11 @@
       </x:c>
       <x:c r="BA31" s="29" t="n">
         <x:f>ROUND(U31*AY31,0)</x:f>
-        <x:v>621275</x:v>
+        <x:v>759246</x:v>
       </x:c>
       <x:c r="BB31" s="29" t="n">
         <x:f>ROUND(U31*AZ31,0)</x:f>
-        <x:v>1053949</x:v>
+        <x:v>1288007</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="72" customHeight="1">
@@ -32484,7 +32664,7 @@
         <x:v>KI-031</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>CP3/render_handoff/manifest_CP3.json</x:v>
+        <x:v>R16_feluletek_fiokok/data/handoff_manifest.json</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
         <x:v>03a</x:v>
@@ -32496,25 +32676,25 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H32" s="19" t="str">
-        <x:v>W01 alsó bútor,5 működő front és120mm süllyesztett szervizbetét</x:v>
+        <x:v>Hat magas fiókos alsó médiafal, eltérő frontszélességekkel</x:v>
       </x:c>
       <x:c r="I32" s="19" t="str">
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J32" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>760H3000S; T51.7601; T60L7040/T60L7140; ZS7M400MU</x:v>
       </x:c>
       <x:c r="K32" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>R16_feluletek_fiokok/data/sources.json; gyártói adatok, nem kereskedői árforrás</x:v>
       </x:c>
       <x:c r="L32" s="19" t="str">
-        <x:v>3600×400×400mm;720+120+4×690</x:v>
+        <x:v>720+450+450+1080+450+450 mm; egy magas fiók frontonként</x:v>
       </x:c>
       <x:c r="M32" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N32" s="19" t="str">
-        <x:v>MAT-02</x:v>
+        <x:v>M16-DRAWER15 / bronzbarna front</x:v>
       </x:c>
       <x:c r="O32" s="19" t="n">
         <x:v>1</x:v>
@@ -32523,7 +32703,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q32" s="20" t="n">
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="R32" s="20" t="n">
         <x:v>0</x:v>
@@ -32536,16 +32716,16 @@
       </x:c>
       <x:c r="U32" s="21" t="n">
         <x:f>O32*Q32+SUM(R32:T32)</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="V32" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W32" s="19" t="str">
-        <x:v>V3.3 tervezői előirányzat 2026-10-26; ajánlat szükséges</x:v>
+        <x:v>R16/data/cost.json és R15/data/cost_allowance.json; bruttó tervezői becslés, nem ajánlat</x:v>
       </x:c>
       <x:c r="X32" s="19" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="Y32" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32569,17 +32749,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF32" s="19" t="str">
-        <x:v>+30000Ft:300mm többlet korpusz/top/front, régi320000×3600/3300≈349091Ft,350000Ft becslés.</x:v>
+        <x:v>760H3000S +T51.7601 +TIPONBLUMOTION S0/S1 +ZS7M400MU; sablonműveletek nyitottak.</x:v>
       </x:c>
       <x:c r="AG32" s="20" t="n">
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="AH32" s="21" t="n">
         <x:f>O32*AG32+SUM(R32:T32)</x:f>
-        <x:v>350000</x:v>
+        <x:v>985000</x:v>
       </x:c>
       <x:c r="AI32" s="19" t="str">
-        <x:v>R05 főváltozat tartalma; korábbi fiók-/aszimmetria-elhagyás nincs automatikusan kiválasztva.</x:v>
+        <x:v>R16 főtartalom. Ugyanez az előirányzat; új önálló gazdaságos változat nincs igazolva.</x:v>
       </x:c>
       <x:c r="AJ32" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -32597,16 +32777,16 @@
         <x:v>TV-02</x:v>
       </x:c>
       <x:c r="AO32" s="1" t="str">
-        <x:v>R10/drawings/W01_R10.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_asztalos_tervcsomag.pdf</x:v>
       </x:c>
       <x:c r="AP32" s="1" t="str">
-        <x:v>R10_TV03*</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_koordinacio.blend; data/parts.json</x:v>
       </x:c>
       <x:c r="AQ32" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
       </x:c>
       <x:c r="AR32" s="1" t="str">
-        <x:v>R02 méretezett ajánlati terv; nem helyszíni méret</x:v>
+        <x:v>Névleges CAD-méret; nem felmérés. Minta, fal és műhelypróba nyitott.</x:v>
       </x:c>
       <x:c r="AS32" s="1" t="str">
         <x:v>HUF</x:v>
@@ -32634,11 +32814,11 @@
       </x:c>
       <x:c r="BA32" s="29" t="n">
         <x:f>ROUND(U32*AY32,0)</x:f>
-        <x:v>280000</x:v>
+        <x:v>788000</x:v>
       </x:c>
       <x:c r="BB32" s="29" t="n">
         <x:f>ROUND(U32*AZ32,0)</x:f>
-        <x:v>490000</x:v>
+        <x:v>1379000</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="72" customHeight="1">
@@ -32652,7 +32832,7 @@
         <x:v>KI-032</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>CP3/render_handoff/manifest_CP3.json</x:v>
+        <x:v>R16_feluletek_fiokok/data/handoff_manifest.json</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
         <x:v>03a</x:v>
@@ -32664,25 +32844,25 @@
         <x:v>Asztalos</x:v>
       </x:c>
       <x:c r="H33" s="19" t="str">
-        <x:v>W01 rögzítés, szerviz és köztes sáv szerelése</x:v>
+        <x:v>W01 rögzítési és műhelyi csomag R15→R16 egyeztetve</x:v>
       </x:c>
       <x:c r="I33" s="19" t="str">
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J33" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>Camar807 IN / MF375 / kötőelemek</x:v>
       </x:c>
       <x:c r="K33" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>R16_feluletek_fiokok/data/sources.json; gyártói adatok, nem kereskedői árforrás</x:v>
       </x:c>
       <x:c r="L33" s="19" t="str">
-        <x:v>R10 TV-01/02/03; tervi4m fal</x:v>
+        <x:v>7 korpuszpár;4 főpanel +bronzbetét</x:v>
       </x:c>
       <x:c r="M33" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N33" s="19" t="str">
-        <x:v>PENDING – műszaki specifikáció szerint</x:v>
+        <x:v>Camar807 IN / MF375 / kötőelemek</x:v>
       </x:c>
       <x:c r="O33" s="19" t="n">
         <x:v>1</x:v>
@@ -32691,7 +32871,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q33" s="20" t="n">
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="R33" s="20" t="n">
         <x:v>0</x:v>
@@ -32704,16 +32884,16 @@
       </x:c>
       <x:c r="U33" s="21" t="n">
         <x:f>O33*Q33+SUM(R33:T33)</x:f>
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="V33" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W33" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03a</x:v>
+        <x:v>R16/data/cost.json és R15/data/cost_allowance.json; bruttó tervezői becslés, nem ajánlat</x:v>
       </x:c>
       <x:c r="X33" s="19" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="Y33" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -32737,17 +32917,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF33" s="19" t="str">
-        <x:v>+15000Ft:3óra többlet szerelési előirányzat×5000Ft. Falteher és szolgáltatáskeresés továbbra ellenőrzendő.</x:v>
+        <x:v>R15 H01–H04,H06,M01–M03:489800 Ft +15000 Ft hetedik Camar pár. Nem adandó újra az R15 összeghez.</x:v>
       </x:c>
       <x:c r="AG33" s="20" t="n">
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="AH33" s="21" t="n">
         <x:f>O33*AG33+SUM(R33:T33)</x:f>
-        <x:v>135000</x:v>
+        <x:v>504800</x:v>
       </x:c>
       <x:c r="AI33" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>R16 főtartalom. Ugyanez az előirányzat; új önálló gazdaságos változat nincs igazolva.</x:v>
       </x:c>
       <x:c r="AJ33" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -32765,16 +32945,16 @@
         <x:v>TV-01; TV-02; TV-03</x:v>
       </x:c>
       <x:c r="AO33" s="1" t="str">
-        <x:v>R10/drawings/W01_R10.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_asztalos_tervcsomag.pdf</x:v>
       </x:c>
       <x:c r="AP33" s="1" t="str">
-        <x:v>R10_TV*</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_koordinacio.blend; data/parts.json</x:v>
       </x:c>
       <x:c r="AQ33" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
       </x:c>
       <x:c r="AR33" s="1" t="str">
-        <x:v>R02 méretezett ajánlati terv; nem helyszíni méret</x:v>
+        <x:v>Névleges CAD-méret; nem felmérés. Minta, fal és műhelypróba nyitott.</x:v>
       </x:c>
       <x:c r="AS33" s="1" t="str">
         <x:v>HUF</x:v>
@@ -32802,11 +32982,11 @@
       </x:c>
       <x:c r="BA33" s="29" t="n">
         <x:f>ROUND(U33*AY33,0)</x:f>
-        <x:v>114750</x:v>
+        <x:v>429080</x:v>
       </x:c>
       <x:c r="BB33" s="29" t="n">
         <x:f>ROUND(U33*AZ33,0)</x:f>
-        <x:v>175500</x:v>
+        <x:v>656240</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
@@ -32988,7 +33168,7 @@
         <x:v>KI-034</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>CP3/render_handoff/manifest_CP3.json</x:v>
+        <x:v>R16_feluletek_fiokok/data/handoff_manifest.json</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
         <x:v>03a</x:v>
@@ -33000,25 +33180,25 @@
         <x:v>Elektronika</x:v>
       </x:c>
       <x:c r="H35" s="19" t="str">
-        <x:v>Teherhordó TV-konzol</x:v>
+        <x:v>Vogel TVM3605 konzol</x:v>
       </x:c>
       <x:c r="I35" s="19" t="str">
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J35" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>3836050 / TVM3605</x:v>
       </x:c>
       <x:c r="K35" s="19" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>R16_feluletek_fiokok/data/sources.json; gyártói adatok, nem kereskedői árforrás</x:v>
       </x:c>
       <x:c r="L35" s="19" t="str">
-        <x:v>TV-03: 2600×36×2330 mm</x:v>
+        <x:v>675×22×428 mm gyári befoglaló</x:v>
       </x:c>
       <x:c r="M35" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N35" s="19" t="str">
-        <x:v>PENDING – műszaki specifikáció szerint</x:v>
+        <x:v>Vogel3836050</x:v>
       </x:c>
       <x:c r="O35" s="19" t="n">
         <x:v>1</x:v>
@@ -33027,7 +33207,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q35" s="20" t="n">
-        <x:v>30000</x:v>
+        <x:v>32000</x:v>
       </x:c>
       <x:c r="R35" s="20" t="n">
         <x:v>0</x:v>
@@ -33040,16 +33220,16 @@
       </x:c>
       <x:c r="U35" s="21" t="n">
         <x:f>O35*Q35+SUM(R35:T35)</x:f>
-        <x:v>30000</x:v>
+        <x:v>32000</x:v>
       </x:c>
       <x:c r="V35" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W35" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 03a</x:v>
+        <x:v>R16/data/cost.json és R15/data/cost_allowance.json; bruttó tervezői becslés, nem ajánlat</x:v>
       </x:c>
       <x:c r="X35" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="Y35" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -33073,17 +33253,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF35" s="19" t="str">
-        <x:v>CP0 becslési csomag: segédanyag és munkadíj a megnevezett tartalom szerint; külön szállítás a 14 sorban. Nem ingyenes szállítás.</x:v>
+        <x:v>R15 H05 kiváltja a régi30000 Ft-os konzolkeretet. Falhorgony szakági ellenőrzés kell.</x:v>
       </x:c>
       <x:c r="AG35" s="20" t="n">
-        <x:v>30000</x:v>
+        <x:v>32000</x:v>
       </x:c>
       <x:c r="AH35" s="21" t="n">
         <x:f>O35*AG35+SUM(R35:T35)</x:f>
-        <x:v>30000</x:v>
+        <x:v>32000</x:v>
       </x:c>
       <x:c r="AI35" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>R16 főtartalom. Ugyanez az előirányzat; új önálló gazdaságos változat nincs igazolva.</x:v>
       </x:c>
       <x:c r="AJ35" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -33101,16 +33281,16 @@
         <x:v>TV-03</x:v>
       </x:c>
       <x:c r="AO35" s="1" t="str">
-        <x:v>CP3/drawings/TV-03_CP3.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_asztalos_tervcsomag.pdf</x:v>
       </x:c>
       <x:c r="AP35" s="1" t="str">
-        <x:v>CP3_TV-03</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_koordinacio.blend; data/parts.json</x:v>
       </x:c>
       <x:c r="AQ35" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
       </x:c>
       <x:c r="AR35" s="1" t="str">
-        <x:v>R02 méretezett ajánlati terv; nem helyszíni méret</x:v>
+        <x:v>Névleges CAD-méret; nem felmérés. Minta, fal és műhelypróba nyitott.</x:v>
       </x:c>
       <x:c r="AS35" s="1" t="str">
         <x:v>HUF</x:v>
@@ -33138,11 +33318,11 @@
       </x:c>
       <x:c r="BA35" s="29" t="n">
         <x:f>ROUND(U35*AY35,0)</x:f>
-        <x:v>25500</x:v>
+        <x:v>27200</x:v>
       </x:c>
       <x:c r="BB35" s="29" t="n">
         <x:f>ROUND(U35*AZ35,0)</x:f>
-        <x:v>39000</x:v>
+        <x:v>41600</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="72" customHeight="1">
@@ -46424,7 +46604,7 @@
         <x:v>KI-114</x:v>
       </x:c>
       <x:c r="D115" s="12" t="str">
-        <x:v>CP3/render_handoff/manifest_CP3.json</x:v>
+        <x:v>R16_feluletek_fiokok/data/handoff_manifest.json</x:v>
       </x:c>
       <x:c r="E115" s="12" t="str">
         <x:v>10</x:v>
@@ -46436,25 +46616,25 @@
         <x:v>Villamos</x:v>
       </x:c>
       <x:c r="H115" s="19" t="str">
-        <x:v>W01 felső, függőleges és alsó vonalfény komplett</x:v>
+        <x:v>W01 hangulatfény +6fiók és2ajtó nyitásérzékelős belső fénye</x:v>
       </x:c>
       <x:c r="I115" s="19" t="str">
         <x:v>UNKNOWN</x:v>
       </x:c>
       <x:c r="J115" s="19" t="str">
-        <x:v>Loox5 LED2074 833.74.308; GL-C-009P jelölt</x:v>
+        <x:v>LPV-150-24; SR-ZG9101FA-DIM; LED3040 833.76.300; sensor833.89.253</x:v>
       </x:c>
       <x:c r="K115" s="19" t="str">
-        <x:v>https://files.hafele.co.uk/catalogfiles/www/25-1010.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/data/sources.json; gyártói adatok, nem kereskedői árforrás</x:v>
       </x:c>
       <x:c r="L115" s="19" t="str">
-        <x:v>Felső2,76m + függőleges2,33m + alsó3,60m=8,69m;10m rendelési keret</x:v>
+        <x:v>102,8 W összes;151,2 W tápegység;8 külön szenzor</x:v>
       </x:c>
       <x:c r="M115" s="19" t="str">
         <x:v>Kyoto Ink: grafit / füstszürke / taupe</x:v>
       </x:c>
       <x:c r="N115" s="19" t="str">
-        <x:v>12V;2700K;9,6W/m;CRI&gt;90;2×60W táp</x:v>
+        <x:v>24V2700K; LPV15024; Sunricher; Loox5</x:v>
       </x:c>
       <x:c r="O115" s="19" t="n">
         <x:v>1</x:v>
@@ -46463,7 +46643,7 @@
         <x:v>csomag</x:v>
       </x:c>
       <x:c r="Q115" s="20" t="n">
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="R115" s="20" t="n">
         <x:v>0</x:v>
@@ -46476,16 +46656,16 @@
       </x:c>
       <x:c r="U115" s="21" t="n">
         <x:f>O115*Q115+SUM(R115:T115)</x:f>
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="V115" s="19" t="str">
         <x:v>előzetes becslés</x:v>
       </x:c>
       <x:c r="W115" s="19" t="str">
-        <x:v>CP0 tervezői előirányzat, nem webshopár; baseline 10</x:v>
+        <x:v>R16/data/cost.json és R15/data/cost_allowance.json; bruttó tervezői becslés, nem ajánlat</x:v>
       </x:c>
       <x:c r="X115" s="19" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="Y115" s="19" t="str">
         <x:v>UNKNOWN – ajánlatban visszaigazolandó</x:v>
@@ -46509,17 +46689,17 @@
         <x:v>PENDING – méret, csatlakozás, anyagminta, teljes bekerülés</x:v>
       </x:c>
       <x:c r="AF115" s="19" t="str">
-        <x:v>R05/data/W01_light_circuit.json:47,328W és31,680W körök. PS-A két párhuzamos ág, mind4m alatt. Hue és hőpróba, PSU/profile SKU nyitott. Tételes45000+25000+24000+24000+12000+20000=150000Ft becslés.</x:v>
+        <x:v>R15 L01–L07:281000 Ft +196000 Ft belső világítás +35000 Ft szervizáthelyezés. Nem dupla tápegység.</x:v>
       </x:c>
       <x:c r="AG115" s="20" t="n">
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="AH115" s="21" t="n">
         <x:f>O115*AG115+SUM(R115:T115)</x:f>
-        <x:v>150000</x:v>
+        <x:v>512000</x:v>
       </x:c>
       <x:c r="AI115" s="19" t="str">
-        <x:v>R05 főváltozat tartalma; korábbi fiók-/aszimmetria-elhagyás nincs automatikusan kiválasztva.</x:v>
+        <x:v>R16 főtartalom. Ugyanez az előirányzat; új önálló gazdaságos változat nincs igazolva.</x:v>
       </x:c>
       <x:c r="AJ115" s="19" t="str">
         <x:v>PENDING</x:v>
@@ -46537,16 +46717,16 @@
         <x:v>TV-03</x:v>
       </x:c>
       <x:c r="AO115" s="1" t="str">
-        <x:v>CP3/drawings/TV-03_CP3.pdf</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_asztalos_tervcsomag.pdf</x:v>
       </x:c>
       <x:c r="AP115" s="1" t="str">
-        <x:v>CP3_TV-03</x:v>
+        <x:v>R16_feluletek_fiokok/rajzok/TV_R16_koordinacio.blend; data/parts.json</x:v>
       </x:c>
       <x:c r="AQ115" s="1" t="str">
         <x:v>egyedi gyártás</x:v>
       </x:c>
       <x:c r="AR115" s="1" t="str">
-        <x:v>R02 méretezett ajánlati terv; nem helyszíni méret</x:v>
+        <x:v>Névleges CAD-méret; nem felmérés. Minta, fal és műhelypróba nyitott.</x:v>
       </x:c>
       <x:c r="AS115" s="1" t="str">
         <x:v>HUF</x:v>
@@ -46574,11 +46754,11 @@
       </x:c>
       <x:c r="BA115" s="29" t="n">
         <x:f>ROUND(U115*AY115,0)</x:f>
-        <x:v>127500</x:v>
+        <x:v>435200</x:v>
       </x:c>
       <x:c r="BB115" s="29" t="n">
         <x:f>ROUND(U115*AZ115,0)</x:f>
-        <x:v>195000</x:v>
+        <x:v>665600</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="72" customHeight="1">
@@ -57214,7 +57394,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf05aa4e9d6a24906"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a8dcef1884f4446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57631,15 +57811,15 @@
       </x:c>
       <x:c r="D16" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A16)</x:f>
-        <x:v>1570500</x:v>
+        <x:v>2747300</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A16)</x:f>
-        <x:v>1570500</x:v>
+        <x:v>2747300</x:v>
       </x:c>
       <x:c r="F16" s="18" t="n">
         <x:f>E16-C16</x:f>
-        <x:v>709500</x:v>
+        <x:v>1886300</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
         <x:v>W01 teljes panelkompozíció és tusgrafikás torony; W01 alsó négyfrontos médiabútor; W01 rögzítés, szerviznyílás, szerelés; TV készülék 65 col célkategória; Teherhordó TV-konzol; HDMI, hálózat, kábelszervezés, audióigény előirányzat</x:v>
@@ -57917,15 +58097,15 @@
       </x:c>
       <x:c r="D27" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$U$2:$U$179,'Elemregiszter'!$E$2:$E$179,A27)</x:f>
-        <x:v>2060360</x:v>
+        <x:v>2422360</x:v>
       </x:c>
       <x:c r="E27" s="18" t="n">
         <x:f>SUMIFS('Elemregiszter'!$AH$2:$AH$179,'Elemregiszter'!$E$2:$E$179,A27)</x:f>
-        <x:v>2060360</x:v>
+        <x:v>2422360</x:v>
       </x:c>
       <x:c r="F27" s="18" t="n">
         <x:f>E27-C27</x:f>
-        <x:v>660360</x:v>
+        <x:v>1022360</x:v>
       </x:c>
       <x:c r="G27" s="19" t="str">
         <x:v>Hue Bridge és hálózati csatlakozás; Hue vezérlők és kapcsolómodulok; Villamos kábel, csatlakozó, doboz és kábelrejtés; Villanyszerelés, mérések, címkézés; Hue programozás, jelenetek, próbaüzem; Somar függeszték és Hue E27; Négy Hue-kompatibilis általános lámpatest/izzó; ML03 általános fény és FL01 falikar, Hue fényforrások; Pultvilágítás szalag, táp, vezérlő, profil és fedél; ML05 Hue mennyezeti lámpa; W01 felső, függőleges és alsó vonalfény komplett; W02/W07 grafikai falmosás komplett; ML06 mennyezeti Hue lámpa; Két éjjeli gömblámpa Hue fényforrással; Fejvég rejtett fénye szalag/táp/profil; Gardróbbelsők funkcionális fénye; Két fürdő mennyezeti és mosdó feletti gyári Hue lámpái; 06.2 két külön rejtett fény és védett szerelvényrendszer; Fürdő tápegységek száraz oldali szervizelhelyezése</x:v>
@@ -58023,15 +58203,15 @@
       </x:c>
       <x:c r="D31" s="18" t="n">
         <x:f>SUM(D2:D30)</x:f>
-        <x:v>22694180</x:v>
+        <x:v>24232980</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
         <x:f>SUM(E2:E30)</x:f>
-        <x:v>22646180</x:v>
+        <x:v>24184980</x:v>
       </x:c>
       <x:c r="F31" s="18" t="n">
         <x:f>SUM(F2:F30)</x:f>
-        <x:v>5035180</x:v>
+        <x:v>6573980</x:v>
       </x:c>
       <x:c r="G31" s="19"/>
     </x:row>

</xml_diff>